<commit_message>
docs(timeline): sync xlsx to 6 Oct 2026 status, forecast date and sorted weekly view
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -977,7 +977,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Status checked 5 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 50%: live API coin grid, category filters and pagination; search pending. Coin details 75%: live API data, estimated values, grade selector and tabs; premium state pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Dashboards, identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
+          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 50%: live API coin grid, category filters and pagination; search pending. Coin details 75%: live API data, estimated values, grade selector and tabs; premium state pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 0%: the unlocked/multi-coin Premium variant has no Figma and no plan flag yet. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="28">
@@ -1010,6 +1010,18 @@
       <c r="B28" t="inlineStr">
         <is>
           <t>Set progress to 100% and record the actual finish in Detailed Timeline column N. Early finishes release dependent work; forecasts use only remaining work and agent availability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sort order</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Detailed Timeline stays in task-ID order (dependency and agent-lane formulas read earlier rows by position, so sorting it would break the schedule). Weekly View is listed by progress (highest first), then task ID, matching the HTML timeline.</t>
         </is>
       </c>
     </row>
@@ -1051,8 +1063,8 @@
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col min="14" max="14" width="26" customWidth="1"/>
-    <col min="15" max="16" width="19" customWidth="1"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -1276,7 +1288,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Account access: Done: welcome, email signup/login, guest sessions, forgot/reset APIs, OTP entry and error states with HTTP-only cookies; pending: Google sign-in (disabled for now) and shared auth entry pop-ups</t>
+          <t>Account access: Done: welcome, email signup/login, guest sessions, forgot/reset APIs, OTP entry and error states with HTTP-only cookies, signed-in redirects and single-history auth steps; pending: Google sign-in (disabled for now) and shared auth entry pop-ups</t>
         </is>
       </c>
       <c r="D4" s="8">
@@ -1317,7 +1329,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N4" s="12"/>
+      <c r="N4" s="12" t="n"/>
       <c r="O4" s="8">
         <f>IF(OR(L4="",L4&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L4/Overview!$B$9,0))</f>
         <v/>
@@ -1338,7 +1350,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Free user dashboard: Dashboard, activity and Coin of the Day entry points</t>
+          <t>Free user dashboard: Done: signed-in /home (Figma 1898:205770) with live marketplace rows, Coin of the Day (free drawer and Premium upsell modal) and a 3-item Global Catalogue widget</t>
         </is>
       </c>
       <c r="D5" s="8">
@@ -1354,7 +1366,7 @@
         <v/>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
         <f>IF(G5&gt;=1,"Done",IF(O5="","Scope pending",IF(E5="","Waiting on dependency",IF(G5&gt;0,"In progress","Planned"))))</f>
@@ -1379,7 +1391,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N5" s="12"/>
+      <c r="N5" s="12" t="n">
+        <v>46301</v>
+      </c>
       <c r="O5" s="8">
         <f>IF(OR(L5="",L5&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L5/Overview!$B$9,0))</f>
         <v/>
@@ -1400,7 +1414,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Premium experience: Premium Coin of the Day, coin details and expert prompt</t>
+          <t>Premium experience: Premium Coin of the Day, coin details and expert prompt; pending: no Figma or plan flag yet for the unlocked/multi-coin Premium variant</t>
         </is>
       </c>
       <c r="D6" s="8">
@@ -1441,7 +1455,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N6" s="12"/>
+      <c r="N6" s="12" t="n"/>
       <c r="O6" s="8">
         <f>IF(OR(L6="",L6&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L6/Overview!$B$9,0))</f>
         <v/>
@@ -1503,7 +1517,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N7" s="12"/>
+      <c r="N7" s="12" t="n"/>
       <c r="O7" s="8">
         <f>IF(OR(L7="",L7&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L7/Overview!$B$9,0))</f>
         <v/>
@@ -1565,7 +1579,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N8" s="12"/>
+      <c r="N8" s="12" t="n"/>
       <c r="O8" s="8">
         <f>IF(OR(L8="",L8&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L8/Overview!$B$9,0))</f>
         <v/>
@@ -1627,7 +1641,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N9" s="12"/>
+      <c r="N9" s="12" t="n"/>
       <c r="O9" s="8">
         <f>IF(OR(L9="",L9&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L9/Overview!$B$9,0))</f>
         <v/>
@@ -1689,7 +1703,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N10" s="12"/>
+      <c r="N10" s="12" t="n"/>
       <c r="O10" s="8">
         <f>IF(OR(L10="",L10&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L10/Overview!$B$9,0))</f>
         <v/>
@@ -1751,7 +1765,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N11" s="12"/>
+      <c r="N11" s="12" t="n"/>
       <c r="O11" s="8">
         <f>IF(OR(L11="",L11&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L11/Overview!$B$9,0))</f>
         <v/>
@@ -1813,7 +1827,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N12" s="12"/>
+      <c r="N12" s="12" t="n"/>
       <c r="O12" s="8">
         <f>IF(OR(L12="",L12&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L12/Overview!$B$9,0))</f>
         <v/>
@@ -1875,7 +1889,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N13" s="12"/>
+      <c r="N13" s="12" t="n"/>
       <c r="O13" s="8">
         <f>IF(OR(L13="",L13&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L13/Overview!$B$9,0))</f>
         <v/>
@@ -2001,7 +2015,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N15" s="12"/>
+      <c r="N15" s="12" t="n"/>
       <c r="O15" s="8">
         <f>IF(OR(L15="",L15&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L15/Overview!$B$9,0))</f>
         <v/>
@@ -2063,7 +2077,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="N16" s="12"/>
+      <c r="N16" s="12" t="n"/>
       <c r="O16" s="8">
         <f>IF(OR(L16="",L16&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L16/Overview!$B$9,0))</f>
         <v/>
@@ -2125,7 +2139,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="N17" s="12"/>
+      <c r="N17" s="12" t="n"/>
       <c r="O17" s="8">
         <f>IF(OR(L17="",L17&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L17/Overview!$B$9,0))</f>
         <v/>
@@ -2187,7 +2201,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N18" s="12"/>
+      <c r="N18" s="12" t="n"/>
       <c r="O18" s="8">
         <f>IF(OR(L18="",L18&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L18/Overview!$B$9,0))</f>
         <v/>
@@ -2249,7 +2263,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N19" s="12"/>
+      <c r="N19" s="12" t="n"/>
       <c r="O19" s="8">
         <f>IF(OR(L19="",L19&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L19/Overview!$B$9,0))</f>
         <v/>
@@ -2311,7 +2325,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N20" s="12"/>
+      <c r="N20" s="12" t="n"/>
       <c r="O20" s="8">
         <f>IF(OR(L20="",L20&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L20/Overview!$B$9,0))</f>
         <v/>
@@ -2373,7 +2387,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N21" s="12"/>
+      <c r="N21" s="12" t="n"/>
       <c r="O21" s="8">
         <f>IF(OR(L21="",L21&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L21/Overview!$B$9,0))</f>
         <v/>
@@ -2435,7 +2449,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N22" s="12"/>
+      <c r="N22" s="12" t="n"/>
       <c r="O22" s="8">
         <f>IF(OR(L22="",L22&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L22/Overview!$B$9,0))</f>
         <v/>
@@ -2497,7 +2511,7 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="N23" s="12"/>
+      <c r="N23" s="12" t="n"/>
       <c r="O23" s="8">
         <f>IF(OR(L23="",L23&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L23/Overview!$B$9,0))</f>
         <v/>
@@ -3011,2479 +3025,2479 @@
     </row>
     <row r="4">
       <c r="A4">
-        <f>'Detailed Timeline'!A4</f>
+        <f>'Detailed Timeline'!A5</f>
         <v/>
       </c>
       <c r="B4">
-        <f>'Detailed Timeline'!B4</f>
+        <f>'Detailed Timeline'!B5</f>
         <v/>
       </c>
       <c r="C4">
-        <f>'Detailed Timeline'!C4</f>
+        <f>'Detailed Timeline'!C5</f>
         <v/>
       </c>
       <c r="D4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(1&gt;='Detailed Timeline'!$I5,1&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(2&gt;='Detailed Timeline'!$I5,2&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="F4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(3&gt;='Detailed Timeline'!$I5,3&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(4&gt;='Detailed Timeline'!$I5,4&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="H4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(5&gt;='Detailed Timeline'!$I5,5&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="I4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(6&gt;='Detailed Timeline'!$I5,6&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="J4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(7&gt;='Detailed Timeline'!$I5,7&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="K4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(8&gt;='Detailed Timeline'!$I5,8&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="L4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(9&gt;='Detailed Timeline'!$I5,9&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="M4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(10&gt;='Detailed Timeline'!$I5,10&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="N4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(11&gt;='Detailed Timeline'!$I5,11&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="O4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(12&gt;='Detailed Timeline'!$I5,12&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="P4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(13&gt;='Detailed Timeline'!$I5,13&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="Q4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(14&gt;='Detailed Timeline'!$I5,14&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="R4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(15&gt;='Detailed Timeline'!$I5,15&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="S4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(16&gt;='Detailed Timeline'!$I5,16&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="T4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(17&gt;='Detailed Timeline'!$I5,17&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="U4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(18&gt;='Detailed Timeline'!$I5,18&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="V4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(19&gt;='Detailed Timeline'!$I5,19&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="W4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(20&gt;='Detailed Timeline'!$I5,20&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="X4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(21&gt;='Detailed Timeline'!$I5,21&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="Y4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(22&gt;='Detailed Timeline'!$I5,22&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="Z4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(23&gt;='Detailed Timeline'!$I5,23&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="AA4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(24&gt;='Detailed Timeline'!$I5,24&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="AB4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(25&gt;='Detailed Timeline'!$I5,25&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
       <c r="AC4" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(26&gt;='Detailed Timeline'!$I5,26&lt;='Detailed Timeline'!$J5),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <f>'Detailed Timeline'!A5</f>
+        <f>'Detailed Timeline'!A14</f>
         <v/>
       </c>
       <c r="B5">
-        <f>'Detailed Timeline'!B5</f>
+        <f>'Detailed Timeline'!B14</f>
         <v/>
       </c>
       <c r="C5">
-        <f>'Detailed Timeline'!C5</f>
+        <f>'Detailed Timeline'!C14</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(1&gt;='Detailed Timeline'!$I5,1&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(2&gt;='Detailed Timeline'!$I5,2&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(3&gt;='Detailed Timeline'!$I5,3&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(4&gt;='Detailed Timeline'!$I5,4&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(5&gt;='Detailed Timeline'!$I5,5&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(6&gt;='Detailed Timeline'!$I5,6&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(7&gt;='Detailed Timeline'!$I5,7&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(8&gt;='Detailed Timeline'!$I5,8&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="L5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(9&gt;='Detailed Timeline'!$I5,9&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="M5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(10&gt;='Detailed Timeline'!$I5,10&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="N5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(11&gt;='Detailed Timeline'!$I5,11&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="O5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(12&gt;='Detailed Timeline'!$I5,12&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="P5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(13&gt;='Detailed Timeline'!$I5,13&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Q5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(14&gt;='Detailed Timeline'!$I5,14&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="R5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(15&gt;='Detailed Timeline'!$I5,15&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="S5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(16&gt;='Detailed Timeline'!$I5,16&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="T5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(17&gt;='Detailed Timeline'!$I5,17&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="U5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(18&gt;='Detailed Timeline'!$I5,18&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="V5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(19&gt;='Detailed Timeline'!$I5,19&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="W5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(20&gt;='Detailed Timeline'!$I5,20&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="X5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(21&gt;='Detailed Timeline'!$I5,21&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Y5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(22&gt;='Detailed Timeline'!$I5,22&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Z5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(23&gt;='Detailed Timeline'!$I5,23&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AA5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(24&gt;='Detailed Timeline'!$I5,24&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AB5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(25&gt;='Detailed Timeline'!$I5,25&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AC5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I5="",'Detailed Timeline'!$J5=""),"",IF(AND(26&gt;='Detailed Timeline'!$I5,26&lt;='Detailed Timeline'!$J5),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <f>'Detailed Timeline'!A6</f>
+        <f>'Detailed Timeline'!A24</f>
         <v/>
       </c>
       <c r="B6">
-        <f>'Detailed Timeline'!B6</f>
+        <f>'Detailed Timeline'!B24</f>
         <v/>
       </c>
       <c r="C6">
-        <f>'Detailed Timeline'!C6</f>
+        <f>'Detailed Timeline'!C24</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="H6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="J6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="K6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="L6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="M6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="N6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="O6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="P6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Q6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="R6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="S6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="T6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="U6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="V6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="W6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="X6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Y6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Z6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AA6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AB6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AC6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <f>'Detailed Timeline'!A7</f>
+        <f>'Detailed Timeline'!A4</f>
         <v/>
       </c>
       <c r="B7">
-        <f>'Detailed Timeline'!B7</f>
+        <f>'Detailed Timeline'!B4</f>
         <v/>
       </c>
       <c r="C7">
-        <f>'Detailed Timeline'!C7</f>
+        <f>'Detailed Timeline'!C4</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(1&gt;='Detailed Timeline'!$I7,1&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(2&gt;='Detailed Timeline'!$I7,2&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(3&gt;='Detailed Timeline'!$I7,3&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(4&gt;='Detailed Timeline'!$I7,4&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(5&gt;='Detailed Timeline'!$I7,5&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(6&gt;='Detailed Timeline'!$I7,6&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="J7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(7&gt;='Detailed Timeline'!$I7,7&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="K7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(8&gt;='Detailed Timeline'!$I7,8&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="L7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(9&gt;='Detailed Timeline'!$I7,9&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="M7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(10&gt;='Detailed Timeline'!$I7,10&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="N7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(11&gt;='Detailed Timeline'!$I7,11&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="O7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(12&gt;='Detailed Timeline'!$I7,12&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="P7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(13&gt;='Detailed Timeline'!$I7,13&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Q7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(14&gt;='Detailed Timeline'!$I7,14&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="R7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(15&gt;='Detailed Timeline'!$I7,15&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="S7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(16&gt;='Detailed Timeline'!$I7,16&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="T7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(17&gt;='Detailed Timeline'!$I7,17&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="U7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(18&gt;='Detailed Timeline'!$I7,18&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="V7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(19&gt;='Detailed Timeline'!$I7,19&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="W7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(20&gt;='Detailed Timeline'!$I7,20&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="X7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(21&gt;='Detailed Timeline'!$I7,21&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Y7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(22&gt;='Detailed Timeline'!$I7,22&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Z7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(23&gt;='Detailed Timeline'!$I7,23&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AA7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(24&gt;='Detailed Timeline'!$I7,24&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AB7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(25&gt;='Detailed Timeline'!$I7,25&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AC7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(26&gt;='Detailed Timeline'!$I7,26&lt;='Detailed Timeline'!$J7),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <f>'Detailed Timeline'!A8</f>
+        <f>'Detailed Timeline'!A12</f>
         <v/>
       </c>
       <c r="B8">
-        <f>'Detailed Timeline'!B8</f>
+        <f>'Detailed Timeline'!B12</f>
         <v/>
       </c>
       <c r="C8">
-        <f>'Detailed Timeline'!C8</f>
+        <f>'Detailed Timeline'!C12</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(1&gt;='Detailed Timeline'!$I8,1&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(2&gt;='Detailed Timeline'!$I8,2&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="F8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(3&gt;='Detailed Timeline'!$I8,3&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(4&gt;='Detailed Timeline'!$I8,4&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="H8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(5&gt;='Detailed Timeline'!$I8,5&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="I8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(6&gt;='Detailed Timeline'!$I8,6&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="J8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(7&gt;='Detailed Timeline'!$I8,7&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="K8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(8&gt;='Detailed Timeline'!$I8,8&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="L8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(9&gt;='Detailed Timeline'!$I8,9&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="M8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(10&gt;='Detailed Timeline'!$I8,10&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="N8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(11&gt;='Detailed Timeline'!$I8,11&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="O8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(12&gt;='Detailed Timeline'!$I8,12&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="P8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(13&gt;='Detailed Timeline'!$I8,13&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Q8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(14&gt;='Detailed Timeline'!$I8,14&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="R8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(15&gt;='Detailed Timeline'!$I8,15&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="S8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(16&gt;='Detailed Timeline'!$I8,16&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="T8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(17&gt;='Detailed Timeline'!$I8,17&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="U8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(18&gt;='Detailed Timeline'!$I8,18&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="V8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(19&gt;='Detailed Timeline'!$I8,19&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="W8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(20&gt;='Detailed Timeline'!$I8,20&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="X8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(21&gt;='Detailed Timeline'!$I8,21&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Y8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(22&gt;='Detailed Timeline'!$I8,22&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Z8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(23&gt;='Detailed Timeline'!$I8,23&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AA8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(24&gt;='Detailed Timeline'!$I8,24&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AB8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(25&gt;='Detailed Timeline'!$I8,25&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AC8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(26&gt;='Detailed Timeline'!$I8,26&lt;='Detailed Timeline'!$J8),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Detailed Timeline'!A9</f>
+        <f>'Detailed Timeline'!A11</f>
         <v/>
       </c>
       <c r="B9">
-        <f>'Detailed Timeline'!B9</f>
+        <f>'Detailed Timeline'!B11</f>
         <v/>
       </c>
       <c r="C9">
-        <f>'Detailed Timeline'!C9</f>
+        <f>'Detailed Timeline'!C11</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(1&gt;='Detailed Timeline'!$I9,1&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(2&gt;='Detailed Timeline'!$I9,2&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(3&gt;='Detailed Timeline'!$I9,3&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(4&gt;='Detailed Timeline'!$I9,4&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(5&gt;='Detailed Timeline'!$I9,5&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(6&gt;='Detailed Timeline'!$I9,6&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="J9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(7&gt;='Detailed Timeline'!$I9,7&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="K9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(8&gt;='Detailed Timeline'!$I9,8&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="L9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(9&gt;='Detailed Timeline'!$I9,9&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="M9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(10&gt;='Detailed Timeline'!$I9,10&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="N9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(11&gt;='Detailed Timeline'!$I9,11&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="O9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(12&gt;='Detailed Timeline'!$I9,12&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="P9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(13&gt;='Detailed Timeline'!$I9,13&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Q9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(14&gt;='Detailed Timeline'!$I9,14&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="R9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(15&gt;='Detailed Timeline'!$I9,15&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="S9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(16&gt;='Detailed Timeline'!$I9,16&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="T9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(17&gt;='Detailed Timeline'!$I9,17&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="U9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(18&gt;='Detailed Timeline'!$I9,18&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="V9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(19&gt;='Detailed Timeline'!$I9,19&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="W9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(20&gt;='Detailed Timeline'!$I9,20&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="X9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(21&gt;='Detailed Timeline'!$I9,21&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Y9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(22&gt;='Detailed Timeline'!$I9,22&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Z9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(23&gt;='Detailed Timeline'!$I9,23&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AA9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(24&gt;='Detailed Timeline'!$I9,24&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AB9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(25&gt;='Detailed Timeline'!$I9,25&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AC9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(26&gt;='Detailed Timeline'!$I9,26&lt;='Detailed Timeline'!$J9),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Detailed Timeline'!A10</f>
+        <f>'Detailed Timeline'!A13</f>
         <v/>
       </c>
       <c r="B10">
-        <f>'Detailed Timeline'!B10</f>
+        <f>'Detailed Timeline'!B13</f>
         <v/>
       </c>
       <c r="C10">
-        <f>'Detailed Timeline'!C10</f>
+        <f>'Detailed Timeline'!C13</f>
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(1&gt;='Detailed Timeline'!$I10,1&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(2&gt;='Detailed Timeline'!$I10,2&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(3&gt;='Detailed Timeline'!$I10,3&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(4&gt;='Detailed Timeline'!$I10,4&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="H10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(5&gt;='Detailed Timeline'!$I10,5&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(6&gt;='Detailed Timeline'!$I10,6&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="J10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(7&gt;='Detailed Timeline'!$I10,7&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="K10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(8&gt;='Detailed Timeline'!$I10,8&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="L10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(9&gt;='Detailed Timeline'!$I10,9&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="M10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(10&gt;='Detailed Timeline'!$I10,10&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="N10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(11&gt;='Detailed Timeline'!$I10,11&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="O10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(12&gt;='Detailed Timeline'!$I10,12&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="P10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(13&gt;='Detailed Timeline'!$I10,13&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Q10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(14&gt;='Detailed Timeline'!$I10,14&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="R10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(15&gt;='Detailed Timeline'!$I10,15&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="S10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(16&gt;='Detailed Timeline'!$I10,16&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="T10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(17&gt;='Detailed Timeline'!$I10,17&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="U10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(18&gt;='Detailed Timeline'!$I10,18&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="V10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(19&gt;='Detailed Timeline'!$I10,19&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="W10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(20&gt;='Detailed Timeline'!$I10,20&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="X10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(21&gt;='Detailed Timeline'!$I10,21&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Y10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(22&gt;='Detailed Timeline'!$I10,22&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Z10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(23&gt;='Detailed Timeline'!$I10,23&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AA10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(24&gt;='Detailed Timeline'!$I10,24&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AB10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(25&gt;='Detailed Timeline'!$I10,25&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AC10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(26&gt;='Detailed Timeline'!$I10,26&lt;='Detailed Timeline'!$J10),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <f>'Detailed Timeline'!A11</f>
+        <f>'Detailed Timeline'!A6</f>
         <v/>
       </c>
       <c r="B11">
-        <f>'Detailed Timeline'!B11</f>
+        <f>'Detailed Timeline'!B6</f>
         <v/>
       </c>
       <c r="C11">
-        <f>'Detailed Timeline'!C11</f>
+        <f>'Detailed Timeline'!C6</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="J11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="K11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="L11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="M11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="N11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="O11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="P11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Q11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="R11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="S11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="T11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="U11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="V11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="W11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="X11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Y11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Z11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AA11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AB11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AC11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <f>'Detailed Timeline'!A12</f>
+        <f>'Detailed Timeline'!A7</f>
         <v/>
       </c>
       <c r="B12">
-        <f>'Detailed Timeline'!B12</f>
+        <f>'Detailed Timeline'!B7</f>
         <v/>
       </c>
       <c r="C12">
-        <f>'Detailed Timeline'!C12</f>
+        <f>'Detailed Timeline'!C7</f>
         <v/>
       </c>
       <c r="D12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(1&gt;='Detailed Timeline'!$I7,1&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(2&gt;='Detailed Timeline'!$I7,2&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="F12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(3&gt;='Detailed Timeline'!$I7,3&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="G12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(4&gt;='Detailed Timeline'!$I7,4&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="H12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(5&gt;='Detailed Timeline'!$I7,5&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="I12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(6&gt;='Detailed Timeline'!$I7,6&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="J12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(7&gt;='Detailed Timeline'!$I7,7&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="K12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(8&gt;='Detailed Timeline'!$I7,8&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="L12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(9&gt;='Detailed Timeline'!$I7,9&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="M12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(10&gt;='Detailed Timeline'!$I7,10&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="N12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(11&gt;='Detailed Timeline'!$I7,11&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="O12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(12&gt;='Detailed Timeline'!$I7,12&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="P12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(13&gt;='Detailed Timeline'!$I7,13&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="Q12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(14&gt;='Detailed Timeline'!$I7,14&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="R12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(15&gt;='Detailed Timeline'!$I7,15&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="S12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(16&gt;='Detailed Timeline'!$I7,16&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="T12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(17&gt;='Detailed Timeline'!$I7,17&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="U12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(18&gt;='Detailed Timeline'!$I7,18&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="V12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(19&gt;='Detailed Timeline'!$I7,19&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="W12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(20&gt;='Detailed Timeline'!$I7,20&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="X12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(21&gt;='Detailed Timeline'!$I7,21&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="Y12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(22&gt;='Detailed Timeline'!$I7,22&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="Z12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(23&gt;='Detailed Timeline'!$I7,23&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="AA12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(24&gt;='Detailed Timeline'!$I7,24&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="AB12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(25&gt;='Detailed Timeline'!$I7,25&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
       <c r="AC12" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I7="",'Detailed Timeline'!$J7=""),"",IF(AND(26&gt;='Detailed Timeline'!$I7,26&lt;='Detailed Timeline'!$J7),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <f>'Detailed Timeline'!A13</f>
+        <f>'Detailed Timeline'!A8</f>
         <v/>
       </c>
       <c r="B13">
-        <f>'Detailed Timeline'!B13</f>
+        <f>'Detailed Timeline'!B8</f>
         <v/>
       </c>
       <c r="C13">
-        <f>'Detailed Timeline'!C13</f>
+        <f>'Detailed Timeline'!C8</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(1&gt;='Detailed Timeline'!$I8,1&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(2&gt;='Detailed Timeline'!$I8,2&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(3&gt;='Detailed Timeline'!$I8,3&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(4&gt;='Detailed Timeline'!$I8,4&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(5&gt;='Detailed Timeline'!$I8,5&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(6&gt;='Detailed Timeline'!$I8,6&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="J13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(7&gt;='Detailed Timeline'!$I8,7&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="K13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(8&gt;='Detailed Timeline'!$I8,8&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="L13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(9&gt;='Detailed Timeline'!$I8,9&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="M13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(10&gt;='Detailed Timeline'!$I8,10&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="N13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(11&gt;='Detailed Timeline'!$I8,11&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="O13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(12&gt;='Detailed Timeline'!$I8,12&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="P13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(13&gt;='Detailed Timeline'!$I8,13&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="Q13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(14&gt;='Detailed Timeline'!$I8,14&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="R13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(15&gt;='Detailed Timeline'!$I8,15&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="S13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(16&gt;='Detailed Timeline'!$I8,16&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="T13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(17&gt;='Detailed Timeline'!$I8,17&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="U13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(18&gt;='Detailed Timeline'!$I8,18&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="V13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(19&gt;='Detailed Timeline'!$I8,19&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="W13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(20&gt;='Detailed Timeline'!$I8,20&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="X13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(21&gt;='Detailed Timeline'!$I8,21&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="Y13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(22&gt;='Detailed Timeline'!$I8,22&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="Z13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(23&gt;='Detailed Timeline'!$I8,23&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="AA13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(24&gt;='Detailed Timeline'!$I8,24&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="AB13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(25&gt;='Detailed Timeline'!$I8,25&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
       <c r="AC13" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I8="",'Detailed Timeline'!$J8=""),"",IF(AND(26&gt;='Detailed Timeline'!$I8,26&lt;='Detailed Timeline'!$J8),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <f>'Detailed Timeline'!A14</f>
+        <f>'Detailed Timeline'!A9</f>
         <v/>
       </c>
       <c r="B14">
-        <f>'Detailed Timeline'!B14</f>
+        <f>'Detailed Timeline'!B9</f>
         <v/>
       </c>
       <c r="C14">
-        <f>'Detailed Timeline'!C14</f>
+        <f>'Detailed Timeline'!C9</f>
         <v/>
       </c>
       <c r="D14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(1&gt;='Detailed Timeline'!$I9,1&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(2&gt;='Detailed Timeline'!$I9,2&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="F14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(3&gt;='Detailed Timeline'!$I9,3&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="G14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(4&gt;='Detailed Timeline'!$I9,4&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="H14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(5&gt;='Detailed Timeline'!$I9,5&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="I14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(6&gt;='Detailed Timeline'!$I9,6&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="J14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(7&gt;='Detailed Timeline'!$I9,7&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="K14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(8&gt;='Detailed Timeline'!$I9,8&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="L14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(9&gt;='Detailed Timeline'!$I9,9&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="M14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(10&gt;='Detailed Timeline'!$I9,10&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="N14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(11&gt;='Detailed Timeline'!$I9,11&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="O14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(12&gt;='Detailed Timeline'!$I9,12&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="P14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(13&gt;='Detailed Timeline'!$I9,13&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="Q14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(14&gt;='Detailed Timeline'!$I9,14&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="R14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(15&gt;='Detailed Timeline'!$I9,15&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="S14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(16&gt;='Detailed Timeline'!$I9,16&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="T14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(17&gt;='Detailed Timeline'!$I9,17&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="U14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(18&gt;='Detailed Timeline'!$I9,18&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="V14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(19&gt;='Detailed Timeline'!$I9,19&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="W14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(20&gt;='Detailed Timeline'!$I9,20&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="X14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(21&gt;='Detailed Timeline'!$I9,21&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="Y14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(22&gt;='Detailed Timeline'!$I9,22&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="Z14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(23&gt;='Detailed Timeline'!$I9,23&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="AA14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(24&gt;='Detailed Timeline'!$I9,24&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="AB14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(25&gt;='Detailed Timeline'!$I9,25&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
       <c r="AC14" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I9="",'Detailed Timeline'!$J9=""),"",IF(AND(26&gt;='Detailed Timeline'!$I9,26&lt;='Detailed Timeline'!$J9),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <f>'Detailed Timeline'!A15</f>
+        <f>'Detailed Timeline'!A10</f>
         <v/>
       </c>
       <c r="B15">
-        <f>'Detailed Timeline'!B15</f>
+        <f>'Detailed Timeline'!B10</f>
         <v/>
       </c>
       <c r="C15">
-        <f>'Detailed Timeline'!C15</f>
+        <f>'Detailed Timeline'!C10</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(1&gt;='Detailed Timeline'!$I15,1&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(1&gt;='Detailed Timeline'!$I10,1&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(2&gt;='Detailed Timeline'!$I15,2&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(2&gt;='Detailed Timeline'!$I10,2&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(3&gt;='Detailed Timeline'!$I15,3&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(3&gt;='Detailed Timeline'!$I10,3&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="G15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(4&gt;='Detailed Timeline'!$I15,4&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(4&gt;='Detailed Timeline'!$I10,4&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="H15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(5&gt;='Detailed Timeline'!$I15,5&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(5&gt;='Detailed Timeline'!$I10,5&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(6&gt;='Detailed Timeline'!$I15,6&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(6&gt;='Detailed Timeline'!$I10,6&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="J15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(7&gt;='Detailed Timeline'!$I15,7&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(7&gt;='Detailed Timeline'!$I10,7&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="K15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(8&gt;='Detailed Timeline'!$I15,8&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(8&gt;='Detailed Timeline'!$I10,8&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="L15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(9&gt;='Detailed Timeline'!$I15,9&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(9&gt;='Detailed Timeline'!$I10,9&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="M15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(10&gt;='Detailed Timeline'!$I15,10&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(10&gt;='Detailed Timeline'!$I10,10&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="N15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(11&gt;='Detailed Timeline'!$I15,11&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(11&gt;='Detailed Timeline'!$I10,11&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="O15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(12&gt;='Detailed Timeline'!$I15,12&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(12&gt;='Detailed Timeline'!$I10,12&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="P15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(13&gt;='Detailed Timeline'!$I15,13&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(13&gt;='Detailed Timeline'!$I10,13&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="Q15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(14&gt;='Detailed Timeline'!$I15,14&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(14&gt;='Detailed Timeline'!$I10,14&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="R15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(15&gt;='Detailed Timeline'!$I15,15&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(15&gt;='Detailed Timeline'!$I10,15&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="S15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(16&gt;='Detailed Timeline'!$I15,16&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(16&gt;='Detailed Timeline'!$I10,16&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="T15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(17&gt;='Detailed Timeline'!$I15,17&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(17&gt;='Detailed Timeline'!$I10,17&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="U15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(18&gt;='Detailed Timeline'!$I15,18&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(18&gt;='Detailed Timeline'!$I10,18&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="V15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(19&gt;='Detailed Timeline'!$I15,19&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(19&gt;='Detailed Timeline'!$I10,19&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="W15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(20&gt;='Detailed Timeline'!$I15,20&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(20&gt;='Detailed Timeline'!$I10,20&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="X15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(21&gt;='Detailed Timeline'!$I15,21&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(21&gt;='Detailed Timeline'!$I10,21&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="Y15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(22&gt;='Detailed Timeline'!$I15,22&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(22&gt;='Detailed Timeline'!$I10,22&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="Z15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(23&gt;='Detailed Timeline'!$I15,23&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(23&gt;='Detailed Timeline'!$I10,23&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="AA15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(24&gt;='Detailed Timeline'!$I15,24&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(24&gt;='Detailed Timeline'!$I10,24&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="AB15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(25&gt;='Detailed Timeline'!$I15,25&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(25&gt;='Detailed Timeline'!$I10,25&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
       <c r="AC15" s="10">
-        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(26&gt;='Detailed Timeline'!$I15,26&lt;='Detailed Timeline'!$J15),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I10="",'Detailed Timeline'!$J10=""),"",IF(AND(26&gt;='Detailed Timeline'!$I10,26&lt;='Detailed Timeline'!$J10),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <f>'Detailed Timeline'!A16</f>
+        <f>'Detailed Timeline'!A15</f>
         <v/>
       </c>
       <c r="B16">
-        <f>'Detailed Timeline'!B16</f>
+        <f>'Detailed Timeline'!B15</f>
         <v/>
       </c>
       <c r="C16">
-        <f>'Detailed Timeline'!C16</f>
+        <f>'Detailed Timeline'!C15</f>
         <v/>
       </c>
       <c r="D16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(1&gt;='Detailed Timeline'!$I16,1&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(1&gt;='Detailed Timeline'!$I15,1&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(2&gt;='Detailed Timeline'!$I16,2&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(2&gt;='Detailed Timeline'!$I15,2&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="F16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(3&gt;='Detailed Timeline'!$I16,3&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(3&gt;='Detailed Timeline'!$I15,3&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="G16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(4&gt;='Detailed Timeline'!$I16,4&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(4&gt;='Detailed Timeline'!$I15,4&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="H16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(5&gt;='Detailed Timeline'!$I16,5&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(5&gt;='Detailed Timeline'!$I15,5&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="I16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(6&gt;='Detailed Timeline'!$I16,6&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(6&gt;='Detailed Timeline'!$I15,6&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="J16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(7&gt;='Detailed Timeline'!$I16,7&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(7&gt;='Detailed Timeline'!$I15,7&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="K16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(8&gt;='Detailed Timeline'!$I16,8&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(8&gt;='Detailed Timeline'!$I15,8&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="L16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(9&gt;='Detailed Timeline'!$I16,9&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(9&gt;='Detailed Timeline'!$I15,9&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="M16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(10&gt;='Detailed Timeline'!$I16,10&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(10&gt;='Detailed Timeline'!$I15,10&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="N16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(11&gt;='Detailed Timeline'!$I16,11&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(11&gt;='Detailed Timeline'!$I15,11&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="O16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(12&gt;='Detailed Timeline'!$I16,12&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(12&gt;='Detailed Timeline'!$I15,12&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="P16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(13&gt;='Detailed Timeline'!$I16,13&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(13&gt;='Detailed Timeline'!$I15,13&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="Q16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(14&gt;='Detailed Timeline'!$I16,14&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(14&gt;='Detailed Timeline'!$I15,14&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="R16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(15&gt;='Detailed Timeline'!$I16,15&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(15&gt;='Detailed Timeline'!$I15,15&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="S16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(16&gt;='Detailed Timeline'!$I16,16&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(16&gt;='Detailed Timeline'!$I15,16&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="T16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(17&gt;='Detailed Timeline'!$I16,17&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(17&gt;='Detailed Timeline'!$I15,17&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="U16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(18&gt;='Detailed Timeline'!$I16,18&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(18&gt;='Detailed Timeline'!$I15,18&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="V16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(19&gt;='Detailed Timeline'!$I16,19&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(19&gt;='Detailed Timeline'!$I15,19&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="W16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(20&gt;='Detailed Timeline'!$I16,20&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(20&gt;='Detailed Timeline'!$I15,20&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="X16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(21&gt;='Detailed Timeline'!$I16,21&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(21&gt;='Detailed Timeline'!$I15,21&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="Y16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(22&gt;='Detailed Timeline'!$I16,22&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(22&gt;='Detailed Timeline'!$I15,22&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="Z16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(23&gt;='Detailed Timeline'!$I16,23&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(23&gt;='Detailed Timeline'!$I15,23&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="AA16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(24&gt;='Detailed Timeline'!$I16,24&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(24&gt;='Detailed Timeline'!$I15,24&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="AB16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(25&gt;='Detailed Timeline'!$I16,25&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(25&gt;='Detailed Timeline'!$I15,25&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
       <c r="AC16" s="10">
-        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(26&gt;='Detailed Timeline'!$I16,26&lt;='Detailed Timeline'!$J16),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I15="",'Detailed Timeline'!$J15=""),"",IF(AND(26&gt;='Detailed Timeline'!$I15,26&lt;='Detailed Timeline'!$J15),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <f>'Detailed Timeline'!A17</f>
+        <f>'Detailed Timeline'!A16</f>
         <v/>
       </c>
       <c r="B17">
-        <f>'Detailed Timeline'!B17</f>
+        <f>'Detailed Timeline'!B16</f>
         <v/>
       </c>
       <c r="C17">
-        <f>'Detailed Timeline'!C17</f>
+        <f>'Detailed Timeline'!C16</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(1&gt;='Detailed Timeline'!$I17,1&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(1&gt;='Detailed Timeline'!$I16,1&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(2&gt;='Detailed Timeline'!$I17,2&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(2&gt;='Detailed Timeline'!$I16,2&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(3&gt;='Detailed Timeline'!$I17,3&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(3&gt;='Detailed Timeline'!$I16,3&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="G17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(4&gt;='Detailed Timeline'!$I17,4&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(4&gt;='Detailed Timeline'!$I16,4&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="H17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(5&gt;='Detailed Timeline'!$I17,5&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(5&gt;='Detailed Timeline'!$I16,5&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(6&gt;='Detailed Timeline'!$I17,6&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(6&gt;='Detailed Timeline'!$I16,6&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="J17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(7&gt;='Detailed Timeline'!$I17,7&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(7&gt;='Detailed Timeline'!$I16,7&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="K17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(8&gt;='Detailed Timeline'!$I17,8&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(8&gt;='Detailed Timeline'!$I16,8&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="L17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(9&gt;='Detailed Timeline'!$I17,9&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(9&gt;='Detailed Timeline'!$I16,9&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="M17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(10&gt;='Detailed Timeline'!$I17,10&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(10&gt;='Detailed Timeline'!$I16,10&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="N17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(11&gt;='Detailed Timeline'!$I17,11&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(11&gt;='Detailed Timeline'!$I16,11&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="O17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(12&gt;='Detailed Timeline'!$I17,12&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(12&gt;='Detailed Timeline'!$I16,12&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="P17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(13&gt;='Detailed Timeline'!$I17,13&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(13&gt;='Detailed Timeline'!$I16,13&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="Q17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(14&gt;='Detailed Timeline'!$I17,14&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(14&gt;='Detailed Timeline'!$I16,14&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="R17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(15&gt;='Detailed Timeline'!$I17,15&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(15&gt;='Detailed Timeline'!$I16,15&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="S17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(16&gt;='Detailed Timeline'!$I17,16&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(16&gt;='Detailed Timeline'!$I16,16&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="T17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(17&gt;='Detailed Timeline'!$I17,17&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(17&gt;='Detailed Timeline'!$I16,17&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="U17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(18&gt;='Detailed Timeline'!$I17,18&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(18&gt;='Detailed Timeline'!$I16,18&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="V17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(19&gt;='Detailed Timeline'!$I17,19&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(19&gt;='Detailed Timeline'!$I16,19&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="W17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(20&gt;='Detailed Timeline'!$I17,20&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(20&gt;='Detailed Timeline'!$I16,20&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="X17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(21&gt;='Detailed Timeline'!$I17,21&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(21&gt;='Detailed Timeline'!$I16,21&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="Y17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(22&gt;='Detailed Timeline'!$I17,22&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(22&gt;='Detailed Timeline'!$I16,22&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="Z17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(23&gt;='Detailed Timeline'!$I17,23&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(23&gt;='Detailed Timeline'!$I16,23&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="AA17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(24&gt;='Detailed Timeline'!$I17,24&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(24&gt;='Detailed Timeline'!$I16,24&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="AB17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(25&gt;='Detailed Timeline'!$I17,25&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(25&gt;='Detailed Timeline'!$I16,25&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
       <c r="AC17" s="10">
-        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(26&gt;='Detailed Timeline'!$I17,26&lt;='Detailed Timeline'!$J17),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I16="",'Detailed Timeline'!$J16=""),"",IF(AND(26&gt;='Detailed Timeline'!$I16,26&lt;='Detailed Timeline'!$J16),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <f>'Detailed Timeline'!A18</f>
+        <f>'Detailed Timeline'!A17</f>
         <v/>
       </c>
       <c r="B18">
-        <f>'Detailed Timeline'!B18</f>
+        <f>'Detailed Timeline'!B17</f>
         <v/>
       </c>
       <c r="C18">
-        <f>'Detailed Timeline'!C18</f>
+        <f>'Detailed Timeline'!C17</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(1&gt;='Detailed Timeline'!$I18,1&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(1&gt;='Detailed Timeline'!$I17,1&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(2&gt;='Detailed Timeline'!$I18,2&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(2&gt;='Detailed Timeline'!$I17,2&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(3&gt;='Detailed Timeline'!$I18,3&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(3&gt;='Detailed Timeline'!$I17,3&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="G18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(4&gt;='Detailed Timeline'!$I18,4&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(4&gt;='Detailed Timeline'!$I17,4&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="H18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(5&gt;='Detailed Timeline'!$I18,5&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(5&gt;='Detailed Timeline'!$I17,5&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="I18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(6&gt;='Detailed Timeline'!$I18,6&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(6&gt;='Detailed Timeline'!$I17,6&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="J18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(7&gt;='Detailed Timeline'!$I18,7&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(7&gt;='Detailed Timeline'!$I17,7&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="K18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(8&gt;='Detailed Timeline'!$I18,8&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(8&gt;='Detailed Timeline'!$I17,8&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="L18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(9&gt;='Detailed Timeline'!$I18,9&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(9&gt;='Detailed Timeline'!$I17,9&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="M18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(10&gt;='Detailed Timeline'!$I18,10&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(10&gt;='Detailed Timeline'!$I17,10&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="N18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(11&gt;='Detailed Timeline'!$I18,11&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(11&gt;='Detailed Timeline'!$I17,11&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="O18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(12&gt;='Detailed Timeline'!$I18,12&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(12&gt;='Detailed Timeline'!$I17,12&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="P18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(13&gt;='Detailed Timeline'!$I18,13&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(13&gt;='Detailed Timeline'!$I17,13&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="Q18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(14&gt;='Detailed Timeline'!$I18,14&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(14&gt;='Detailed Timeline'!$I17,14&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="R18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(15&gt;='Detailed Timeline'!$I18,15&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(15&gt;='Detailed Timeline'!$I17,15&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="S18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(16&gt;='Detailed Timeline'!$I18,16&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(16&gt;='Detailed Timeline'!$I17,16&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="T18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(17&gt;='Detailed Timeline'!$I18,17&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(17&gt;='Detailed Timeline'!$I17,17&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="U18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(18&gt;='Detailed Timeline'!$I18,18&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(18&gt;='Detailed Timeline'!$I17,18&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="V18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(19&gt;='Detailed Timeline'!$I18,19&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(19&gt;='Detailed Timeline'!$I17,19&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="W18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(20&gt;='Detailed Timeline'!$I18,20&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(20&gt;='Detailed Timeline'!$I17,20&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="X18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(21&gt;='Detailed Timeline'!$I18,21&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(21&gt;='Detailed Timeline'!$I17,21&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="Y18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(22&gt;='Detailed Timeline'!$I18,22&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(22&gt;='Detailed Timeline'!$I17,22&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="Z18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(23&gt;='Detailed Timeline'!$I18,23&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(23&gt;='Detailed Timeline'!$I17,23&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="AA18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(24&gt;='Detailed Timeline'!$I18,24&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(24&gt;='Detailed Timeline'!$I17,24&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="AB18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(25&gt;='Detailed Timeline'!$I18,25&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(25&gt;='Detailed Timeline'!$I17,25&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
       <c r="AC18" s="10">
-        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(26&gt;='Detailed Timeline'!$I18,26&lt;='Detailed Timeline'!$J18),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I17="",'Detailed Timeline'!$J17=""),"",IF(AND(26&gt;='Detailed Timeline'!$I17,26&lt;='Detailed Timeline'!$J17),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <f>'Detailed Timeline'!A19</f>
+        <f>'Detailed Timeline'!A18</f>
         <v/>
       </c>
       <c r="B19">
-        <f>'Detailed Timeline'!B19</f>
+        <f>'Detailed Timeline'!B18</f>
         <v/>
       </c>
       <c r="C19">
-        <f>'Detailed Timeline'!C19</f>
+        <f>'Detailed Timeline'!C18</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(1&gt;='Detailed Timeline'!$I19,1&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(1&gt;='Detailed Timeline'!$I18,1&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(2&gt;='Detailed Timeline'!$I19,2&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(2&gt;='Detailed Timeline'!$I18,2&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(3&gt;='Detailed Timeline'!$I19,3&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(3&gt;='Detailed Timeline'!$I18,3&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(4&gt;='Detailed Timeline'!$I19,4&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(4&gt;='Detailed Timeline'!$I18,4&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(5&gt;='Detailed Timeline'!$I19,5&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(5&gt;='Detailed Timeline'!$I18,5&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(6&gt;='Detailed Timeline'!$I19,6&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(6&gt;='Detailed Timeline'!$I18,6&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="J19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(7&gt;='Detailed Timeline'!$I19,7&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(7&gt;='Detailed Timeline'!$I18,7&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="K19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(8&gt;='Detailed Timeline'!$I19,8&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(8&gt;='Detailed Timeline'!$I18,8&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="L19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(9&gt;='Detailed Timeline'!$I19,9&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(9&gt;='Detailed Timeline'!$I18,9&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="M19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(10&gt;='Detailed Timeline'!$I19,10&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(10&gt;='Detailed Timeline'!$I18,10&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="N19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(11&gt;='Detailed Timeline'!$I19,11&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(11&gt;='Detailed Timeline'!$I18,11&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="O19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(12&gt;='Detailed Timeline'!$I19,12&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(12&gt;='Detailed Timeline'!$I18,12&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="P19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(13&gt;='Detailed Timeline'!$I19,13&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(13&gt;='Detailed Timeline'!$I18,13&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="Q19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(14&gt;='Detailed Timeline'!$I19,14&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(14&gt;='Detailed Timeline'!$I18,14&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="R19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(15&gt;='Detailed Timeline'!$I19,15&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(15&gt;='Detailed Timeline'!$I18,15&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="S19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(16&gt;='Detailed Timeline'!$I19,16&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(16&gt;='Detailed Timeline'!$I18,16&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="T19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(17&gt;='Detailed Timeline'!$I19,17&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(17&gt;='Detailed Timeline'!$I18,17&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="U19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(18&gt;='Detailed Timeline'!$I19,18&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(18&gt;='Detailed Timeline'!$I18,18&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="V19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(19&gt;='Detailed Timeline'!$I19,19&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(19&gt;='Detailed Timeline'!$I18,19&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="W19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(20&gt;='Detailed Timeline'!$I19,20&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(20&gt;='Detailed Timeline'!$I18,20&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="X19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(21&gt;='Detailed Timeline'!$I19,21&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(21&gt;='Detailed Timeline'!$I18,21&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="Y19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(22&gt;='Detailed Timeline'!$I19,22&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(22&gt;='Detailed Timeline'!$I18,22&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="Z19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(23&gt;='Detailed Timeline'!$I19,23&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(23&gt;='Detailed Timeline'!$I18,23&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="AA19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(24&gt;='Detailed Timeline'!$I19,24&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(24&gt;='Detailed Timeline'!$I18,24&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="AB19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(25&gt;='Detailed Timeline'!$I19,25&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(25&gt;='Detailed Timeline'!$I18,25&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
       <c r="AC19" s="10">
-        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(26&gt;='Detailed Timeline'!$I19,26&lt;='Detailed Timeline'!$J19),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I18="",'Detailed Timeline'!$J18=""),"",IF(AND(26&gt;='Detailed Timeline'!$I18,26&lt;='Detailed Timeline'!$J18),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <f>'Detailed Timeline'!A20</f>
+        <f>'Detailed Timeline'!A19</f>
         <v/>
       </c>
       <c r="B20">
-        <f>'Detailed Timeline'!B20</f>
+        <f>'Detailed Timeline'!B19</f>
         <v/>
       </c>
       <c r="C20">
-        <f>'Detailed Timeline'!C20</f>
+        <f>'Detailed Timeline'!C19</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(1&gt;='Detailed Timeline'!$I20,1&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(1&gt;='Detailed Timeline'!$I19,1&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(2&gt;='Detailed Timeline'!$I20,2&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(2&gt;='Detailed Timeline'!$I19,2&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(3&gt;='Detailed Timeline'!$I20,3&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(3&gt;='Detailed Timeline'!$I19,3&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="G20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(4&gt;='Detailed Timeline'!$I20,4&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(4&gt;='Detailed Timeline'!$I19,4&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="H20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(5&gt;='Detailed Timeline'!$I20,5&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(5&gt;='Detailed Timeline'!$I19,5&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="I20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(6&gt;='Detailed Timeline'!$I20,6&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(6&gt;='Detailed Timeline'!$I19,6&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="J20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(7&gt;='Detailed Timeline'!$I20,7&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(7&gt;='Detailed Timeline'!$I19,7&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="K20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(8&gt;='Detailed Timeline'!$I20,8&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(8&gt;='Detailed Timeline'!$I19,8&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="L20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(9&gt;='Detailed Timeline'!$I20,9&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(9&gt;='Detailed Timeline'!$I19,9&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="M20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(10&gt;='Detailed Timeline'!$I20,10&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(10&gt;='Detailed Timeline'!$I19,10&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="N20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(11&gt;='Detailed Timeline'!$I20,11&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(11&gt;='Detailed Timeline'!$I19,11&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="O20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(12&gt;='Detailed Timeline'!$I20,12&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(12&gt;='Detailed Timeline'!$I19,12&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="P20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(13&gt;='Detailed Timeline'!$I20,13&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(13&gt;='Detailed Timeline'!$I19,13&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="Q20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(14&gt;='Detailed Timeline'!$I20,14&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(14&gt;='Detailed Timeline'!$I19,14&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="R20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(15&gt;='Detailed Timeline'!$I20,15&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(15&gt;='Detailed Timeline'!$I19,15&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="S20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(16&gt;='Detailed Timeline'!$I20,16&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(16&gt;='Detailed Timeline'!$I19,16&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="T20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(17&gt;='Detailed Timeline'!$I20,17&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(17&gt;='Detailed Timeline'!$I19,17&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="U20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(18&gt;='Detailed Timeline'!$I20,18&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(18&gt;='Detailed Timeline'!$I19,18&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="V20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(19&gt;='Detailed Timeline'!$I20,19&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(19&gt;='Detailed Timeline'!$I19,19&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="W20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(20&gt;='Detailed Timeline'!$I20,20&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(20&gt;='Detailed Timeline'!$I19,20&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="X20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(21&gt;='Detailed Timeline'!$I20,21&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(21&gt;='Detailed Timeline'!$I19,21&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="Y20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(22&gt;='Detailed Timeline'!$I20,22&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(22&gt;='Detailed Timeline'!$I19,22&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="Z20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(23&gt;='Detailed Timeline'!$I20,23&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(23&gt;='Detailed Timeline'!$I19,23&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="AA20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(24&gt;='Detailed Timeline'!$I20,24&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(24&gt;='Detailed Timeline'!$I19,24&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="AB20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(25&gt;='Detailed Timeline'!$I20,25&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(25&gt;='Detailed Timeline'!$I19,25&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
       <c r="AC20" s="10">
-        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(26&gt;='Detailed Timeline'!$I20,26&lt;='Detailed Timeline'!$J20),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I19="",'Detailed Timeline'!$J19=""),"",IF(AND(26&gt;='Detailed Timeline'!$I19,26&lt;='Detailed Timeline'!$J19),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <f>'Detailed Timeline'!A21</f>
+        <f>'Detailed Timeline'!A20</f>
         <v/>
       </c>
       <c r="B21">
-        <f>'Detailed Timeline'!B21</f>
+        <f>'Detailed Timeline'!B20</f>
         <v/>
       </c>
       <c r="C21">
-        <f>'Detailed Timeline'!C21</f>
+        <f>'Detailed Timeline'!C20</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(1&gt;='Detailed Timeline'!$I21,1&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(1&gt;='Detailed Timeline'!$I20,1&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(2&gt;='Detailed Timeline'!$I21,2&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(2&gt;='Detailed Timeline'!$I20,2&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(3&gt;='Detailed Timeline'!$I21,3&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(3&gt;='Detailed Timeline'!$I20,3&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="G21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(4&gt;='Detailed Timeline'!$I21,4&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(4&gt;='Detailed Timeline'!$I20,4&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="H21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(5&gt;='Detailed Timeline'!$I21,5&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(5&gt;='Detailed Timeline'!$I20,5&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(6&gt;='Detailed Timeline'!$I21,6&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(6&gt;='Detailed Timeline'!$I20,6&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="J21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(7&gt;='Detailed Timeline'!$I21,7&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(7&gt;='Detailed Timeline'!$I20,7&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="K21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(8&gt;='Detailed Timeline'!$I21,8&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(8&gt;='Detailed Timeline'!$I20,8&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="L21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(9&gt;='Detailed Timeline'!$I21,9&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(9&gt;='Detailed Timeline'!$I20,9&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="M21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(10&gt;='Detailed Timeline'!$I21,10&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(10&gt;='Detailed Timeline'!$I20,10&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="N21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(11&gt;='Detailed Timeline'!$I21,11&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(11&gt;='Detailed Timeline'!$I20,11&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="O21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(12&gt;='Detailed Timeline'!$I21,12&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(12&gt;='Detailed Timeline'!$I20,12&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="P21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(13&gt;='Detailed Timeline'!$I21,13&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(13&gt;='Detailed Timeline'!$I20,13&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="Q21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(14&gt;='Detailed Timeline'!$I21,14&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(14&gt;='Detailed Timeline'!$I20,14&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="R21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(15&gt;='Detailed Timeline'!$I21,15&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(15&gt;='Detailed Timeline'!$I20,15&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="S21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(16&gt;='Detailed Timeline'!$I21,16&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(16&gt;='Detailed Timeline'!$I20,16&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="T21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(17&gt;='Detailed Timeline'!$I21,17&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(17&gt;='Detailed Timeline'!$I20,17&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="U21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(18&gt;='Detailed Timeline'!$I21,18&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(18&gt;='Detailed Timeline'!$I20,18&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="V21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(19&gt;='Detailed Timeline'!$I21,19&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(19&gt;='Detailed Timeline'!$I20,19&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="W21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(20&gt;='Detailed Timeline'!$I21,20&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(20&gt;='Detailed Timeline'!$I20,20&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="X21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(21&gt;='Detailed Timeline'!$I21,21&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(21&gt;='Detailed Timeline'!$I20,21&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="Y21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(22&gt;='Detailed Timeline'!$I21,22&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(22&gt;='Detailed Timeline'!$I20,22&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="Z21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(23&gt;='Detailed Timeline'!$I21,23&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(23&gt;='Detailed Timeline'!$I20,23&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="AA21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(24&gt;='Detailed Timeline'!$I21,24&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(24&gt;='Detailed Timeline'!$I20,24&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="AB21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(25&gt;='Detailed Timeline'!$I21,25&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(25&gt;='Detailed Timeline'!$I20,25&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
       <c r="AC21" s="10">
-        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(26&gt;='Detailed Timeline'!$I21,26&lt;='Detailed Timeline'!$J21),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I20="",'Detailed Timeline'!$J20=""),"",IF(AND(26&gt;='Detailed Timeline'!$I20,26&lt;='Detailed Timeline'!$J20),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <f>'Detailed Timeline'!A22</f>
+        <f>'Detailed Timeline'!A21</f>
         <v/>
       </c>
       <c r="B22">
-        <f>'Detailed Timeline'!B22</f>
+        <f>'Detailed Timeline'!B21</f>
         <v/>
       </c>
       <c r="C22">
-        <f>'Detailed Timeline'!C22</f>
+        <f>'Detailed Timeline'!C21</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(1&gt;='Detailed Timeline'!$I22,1&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(1&gt;='Detailed Timeline'!$I21,1&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(2&gt;='Detailed Timeline'!$I22,2&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(2&gt;='Detailed Timeline'!$I21,2&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(3&gt;='Detailed Timeline'!$I22,3&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(3&gt;='Detailed Timeline'!$I21,3&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="G22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(4&gt;='Detailed Timeline'!$I22,4&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(4&gt;='Detailed Timeline'!$I21,4&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="H22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(5&gt;='Detailed Timeline'!$I22,5&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(5&gt;='Detailed Timeline'!$I21,5&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="I22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(6&gt;='Detailed Timeline'!$I22,6&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(6&gt;='Detailed Timeline'!$I21,6&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="J22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(7&gt;='Detailed Timeline'!$I22,7&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(7&gt;='Detailed Timeline'!$I21,7&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="K22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(8&gt;='Detailed Timeline'!$I22,8&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(8&gt;='Detailed Timeline'!$I21,8&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="L22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(9&gt;='Detailed Timeline'!$I22,9&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(9&gt;='Detailed Timeline'!$I21,9&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="M22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(10&gt;='Detailed Timeline'!$I22,10&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(10&gt;='Detailed Timeline'!$I21,10&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="N22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(11&gt;='Detailed Timeline'!$I22,11&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(11&gt;='Detailed Timeline'!$I21,11&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="O22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(12&gt;='Detailed Timeline'!$I22,12&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(12&gt;='Detailed Timeline'!$I21,12&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="P22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(13&gt;='Detailed Timeline'!$I22,13&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(13&gt;='Detailed Timeline'!$I21,13&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="Q22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(14&gt;='Detailed Timeline'!$I22,14&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(14&gt;='Detailed Timeline'!$I21,14&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="R22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(15&gt;='Detailed Timeline'!$I22,15&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(15&gt;='Detailed Timeline'!$I21,15&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="S22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(16&gt;='Detailed Timeline'!$I22,16&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(16&gt;='Detailed Timeline'!$I21,16&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="T22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(17&gt;='Detailed Timeline'!$I22,17&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(17&gt;='Detailed Timeline'!$I21,17&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="U22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(18&gt;='Detailed Timeline'!$I22,18&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(18&gt;='Detailed Timeline'!$I21,18&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="V22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(19&gt;='Detailed Timeline'!$I22,19&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(19&gt;='Detailed Timeline'!$I21,19&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="W22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(20&gt;='Detailed Timeline'!$I22,20&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(20&gt;='Detailed Timeline'!$I21,20&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="X22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(21&gt;='Detailed Timeline'!$I22,21&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(21&gt;='Detailed Timeline'!$I21,21&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="Y22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(22&gt;='Detailed Timeline'!$I22,22&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(22&gt;='Detailed Timeline'!$I21,22&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="Z22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(23&gt;='Detailed Timeline'!$I22,23&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(23&gt;='Detailed Timeline'!$I21,23&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="AA22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(24&gt;='Detailed Timeline'!$I22,24&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(24&gt;='Detailed Timeline'!$I21,24&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="AB22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(25&gt;='Detailed Timeline'!$I22,25&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(25&gt;='Detailed Timeline'!$I21,25&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
       <c r="AC22" s="10">
-        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(26&gt;='Detailed Timeline'!$I22,26&lt;='Detailed Timeline'!$J22),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I21="",'Detailed Timeline'!$J21=""),"",IF(AND(26&gt;='Detailed Timeline'!$I21,26&lt;='Detailed Timeline'!$J21),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <f>'Detailed Timeline'!A23</f>
+        <f>'Detailed Timeline'!A22</f>
         <v/>
       </c>
       <c r="B23">
-        <f>'Detailed Timeline'!B23</f>
+        <f>'Detailed Timeline'!B22</f>
         <v/>
       </c>
       <c r="C23">
-        <f>'Detailed Timeline'!C23</f>
+        <f>'Detailed Timeline'!C22</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(1&gt;='Detailed Timeline'!$I23,1&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(1&gt;='Detailed Timeline'!$I22,1&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(2&gt;='Detailed Timeline'!$I23,2&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(2&gt;='Detailed Timeline'!$I22,2&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(3&gt;='Detailed Timeline'!$I23,3&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(3&gt;='Detailed Timeline'!$I22,3&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="G23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(4&gt;='Detailed Timeline'!$I23,4&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(4&gt;='Detailed Timeline'!$I22,4&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="H23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(5&gt;='Detailed Timeline'!$I23,5&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(5&gt;='Detailed Timeline'!$I22,5&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(6&gt;='Detailed Timeline'!$I23,6&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(6&gt;='Detailed Timeline'!$I22,6&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="J23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(7&gt;='Detailed Timeline'!$I23,7&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(7&gt;='Detailed Timeline'!$I22,7&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="K23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(8&gt;='Detailed Timeline'!$I23,8&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(8&gt;='Detailed Timeline'!$I22,8&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="L23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(9&gt;='Detailed Timeline'!$I23,9&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(9&gt;='Detailed Timeline'!$I22,9&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="M23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(10&gt;='Detailed Timeline'!$I23,10&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(10&gt;='Detailed Timeline'!$I22,10&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="N23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(11&gt;='Detailed Timeline'!$I23,11&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(11&gt;='Detailed Timeline'!$I22,11&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="O23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(12&gt;='Detailed Timeline'!$I23,12&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(12&gt;='Detailed Timeline'!$I22,12&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="P23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(13&gt;='Detailed Timeline'!$I23,13&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(13&gt;='Detailed Timeline'!$I22,13&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="Q23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(14&gt;='Detailed Timeline'!$I23,14&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(14&gt;='Detailed Timeline'!$I22,14&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="R23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(15&gt;='Detailed Timeline'!$I23,15&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(15&gt;='Detailed Timeline'!$I22,15&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="S23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(16&gt;='Detailed Timeline'!$I23,16&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(16&gt;='Detailed Timeline'!$I22,16&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="T23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(17&gt;='Detailed Timeline'!$I23,17&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(17&gt;='Detailed Timeline'!$I22,17&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="U23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(18&gt;='Detailed Timeline'!$I23,18&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(18&gt;='Detailed Timeline'!$I22,18&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="V23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(19&gt;='Detailed Timeline'!$I23,19&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(19&gt;='Detailed Timeline'!$I22,19&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="W23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(20&gt;='Detailed Timeline'!$I23,20&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(20&gt;='Detailed Timeline'!$I22,20&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="X23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(21&gt;='Detailed Timeline'!$I23,21&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(21&gt;='Detailed Timeline'!$I22,21&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="Y23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(22&gt;='Detailed Timeline'!$I23,22&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(22&gt;='Detailed Timeline'!$I22,22&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="Z23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(23&gt;='Detailed Timeline'!$I23,23&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(23&gt;='Detailed Timeline'!$I22,23&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="AA23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(24&gt;='Detailed Timeline'!$I23,24&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(24&gt;='Detailed Timeline'!$I22,24&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="AB23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(25&gt;='Detailed Timeline'!$I23,25&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(25&gt;='Detailed Timeline'!$I22,25&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
       <c r="AC23" s="10">
-        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(26&gt;='Detailed Timeline'!$I23,26&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I22="",'Detailed Timeline'!$J22=""),"",IF(AND(26&gt;='Detailed Timeline'!$I22,26&lt;='Detailed Timeline'!$J22),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <f>'Detailed Timeline'!A24</f>
+        <f>'Detailed Timeline'!A23</f>
         <v/>
       </c>
       <c r="B24">
-        <f>'Detailed Timeline'!B24</f>
+        <f>'Detailed Timeline'!B23</f>
         <v/>
       </c>
       <c r="C24">
-        <f>'Detailed Timeline'!C24</f>
+        <f>'Detailed Timeline'!C23</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(1&gt;='Detailed Timeline'!$I23,1&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(2&gt;='Detailed Timeline'!$I23,2&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(3&gt;='Detailed Timeline'!$I23,3&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="G24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(4&gt;='Detailed Timeline'!$I23,4&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="H24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(5&gt;='Detailed Timeline'!$I23,5&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="I24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(6&gt;='Detailed Timeline'!$I23,6&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="J24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(7&gt;='Detailed Timeline'!$I23,7&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="K24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(8&gt;='Detailed Timeline'!$I23,8&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="L24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(9&gt;='Detailed Timeline'!$I23,9&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="M24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(10&gt;='Detailed Timeline'!$I23,10&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="N24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(11&gt;='Detailed Timeline'!$I23,11&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="O24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(12&gt;='Detailed Timeline'!$I23,12&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="P24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(13&gt;='Detailed Timeline'!$I23,13&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="Q24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(14&gt;='Detailed Timeline'!$I23,14&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="R24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(15&gt;='Detailed Timeline'!$I23,15&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="S24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(16&gt;='Detailed Timeline'!$I23,16&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="T24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(17&gt;='Detailed Timeline'!$I23,17&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="U24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(18&gt;='Detailed Timeline'!$I23,18&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="V24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(19&gt;='Detailed Timeline'!$I23,19&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="W24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(20&gt;='Detailed Timeline'!$I23,20&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="X24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(21&gt;='Detailed Timeline'!$I23,21&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="Y24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(22&gt;='Detailed Timeline'!$I23,22&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="Z24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(23&gt;='Detailed Timeline'!$I23,23&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="AA24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(24&gt;='Detailed Timeline'!$I23,24&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="AB24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(25&gt;='Detailed Timeline'!$I23,25&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
       <c r="AC24" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(26&gt;='Detailed Timeline'!$I23,26&lt;='Detailed Timeline'!$J23),"■",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(timeline): task 5 Premium experience at 60%
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -977,7 +977,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 50%: live API coin grid, category filters and pagination; search pending. Coin details 75%: live API data, estimated values, grade selector and tabs; premium state pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 0%: the unlocked/multi-coin Premium variant has no Figma and no plan flag yet. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
+          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 50%: live API coin grid, category filters and pagination; search pending. Coin details 75%: live API data, estimated values, grade selector and tabs; premium state pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 60% (6 Oct): Premium home variant (1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426) are built and verified against Figma, but only reachable through a dev-only ?premium=1 preview because the API documents no plan/entitlement flag; Premium coin details state and expert prompt remain pending. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Premium experience: Premium Coin of the Day, coin details and expert prompt; pending: no Figma or plan flag yet for the unlocked/multi-coin Premium variant</t>
+          <t>Premium experience: Done: Premium home variant (Figma 1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426), shown via the dev-only ?premium=1 preview; pending: real plan/entitlement flag from the API, Premium coin details state and expert prompt</t>
         </is>
       </c>
       <c r="D6" s="8">
@@ -1430,7 +1430,7 @@
         <v/>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="H6">
         <f>IF(G6&gt;=1,"Done",IF(O6="","Scope pending",IF(E6="","Waiting on dependency",IF(G6&gt;0,"In progress","Planned"))))</f>
@@ -3615,355 +3615,355 @@
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Detailed Timeline'!A11</f>
+        <f>'Detailed Timeline'!A6</f>
         <v/>
       </c>
       <c r="B9">
-        <f>'Detailed Timeline'!B11</f>
+        <f>'Detailed Timeline'!B6</f>
         <v/>
       </c>
       <c r="C9">
-        <f>'Detailed Timeline'!C11</f>
+        <f>'Detailed Timeline'!C6</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="J9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="K9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="L9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="M9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="N9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="O9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="P9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Q9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="R9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="S9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="T9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="U9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="V9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="W9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="X9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Y9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Z9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AA9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AB9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AC9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Detailed Timeline'!A13</f>
+        <f>'Detailed Timeline'!A11</f>
         <v/>
       </c>
       <c r="B10">
-        <f>'Detailed Timeline'!B13</f>
+        <f>'Detailed Timeline'!B11</f>
         <v/>
       </c>
       <c r="C10">
-        <f>'Detailed Timeline'!C13</f>
+        <f>'Detailed Timeline'!C11</f>
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="H10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="J10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="K10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="L10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="M10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="N10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="O10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="P10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Q10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="R10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="S10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="T10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="U10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="V10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="W10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="X10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Y10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Z10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AA10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AB10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AC10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <f>'Detailed Timeline'!A6</f>
+        <f>'Detailed Timeline'!A13</f>
         <v/>
       </c>
       <c r="B11">
-        <f>'Detailed Timeline'!B6</f>
+        <f>'Detailed Timeline'!B13</f>
         <v/>
       </c>
       <c r="C11">
-        <f>'Detailed Timeline'!C6</f>
+        <f>'Detailed Timeline'!C13</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="J11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="K11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="L11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="M11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="N11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="O11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="P11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Q11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="R11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="S11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="T11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="U11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="V11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="W11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="X11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Y11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Z11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AA11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AB11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AC11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(timeline): catalogue browse 100%, coin details note
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -977,7 +977,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 50%: live API coin grid, category filters and pagination; search pending. Coin details 75%: live API data, estimated values, grade selector and tabs; premium state pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 60% (6 Oct): Premium home variant (1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426) are built and verified against Figma, but only reachable through a dev-only ?premium=1 preview because the API documents no plan/entitlement flag; Premium coin details state and expert prompt remain pending. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
+          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 100% (6 Oct): live API coin grid, category filters, pagination and name search; the search box is not in Figma (reuses the dashboard search pill) and the API only matches whole coin names, so partial words return nothing. Coin details 75%: live API data, estimated values, grade selector and tabs; the premium state has no Figma node, so it stays pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 60% (6 Oct): Premium home variant (1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426) are built and verified against Figma, but only reachable through a dev-only ?premium=1 preview because the API documents no plan/entitlement flag; Premium coin details state and expert prompt remain pending. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Browse catalogue: Done: live API coin grid, category filters and pagination; search pending</t>
+          <t>Browse catalogue: Done: live API coin grid, category filters, pagination and name search (?q=, composes with category filters; the API matches whole coin names only; search UI is not in Figma, built on the dashboard search pill)</t>
         </is>
       </c>
       <c r="D11" s="8">
@@ -1740,7 +1740,7 @@
         <v/>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <f>IF(G11&gt;=1,"Done",IF(O11="","Scope pending",IF(E11="","Waiting on dependency",IF(G11&gt;0,"In progress","Planned"))))</f>
@@ -1765,7 +1765,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N11" s="12" t="n"/>
+      <c r="N11" s="12" t="n">
+        <v>46301</v>
+      </c>
       <c r="O11" s="8">
         <f>IF(OR(L11="",L11&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L11/Overview!$B$9,0))</f>
         <v/>
@@ -1786,7 +1788,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Coin details: Done: live coin information, estimated value, grades and tabs; premium state pending</t>
+          <t>Coin details: Done: live coin information, estimated value, grades and tabs; premium state pending (no Figma node exists for it)</t>
         </is>
       </c>
       <c r="D12" s="8">
@@ -3143,709 +3145,709 @@
     </row>
     <row r="5">
       <c r="A5">
-        <f>'Detailed Timeline'!A14</f>
+        <f>'Detailed Timeline'!A11</f>
         <v/>
       </c>
       <c r="B5">
-        <f>'Detailed Timeline'!B14</f>
+        <f>'Detailed Timeline'!B11</f>
         <v/>
       </c>
       <c r="C5">
-        <f>'Detailed Timeline'!C14</f>
+        <f>'Detailed Timeline'!C11</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="L5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="M5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="N5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="O5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="P5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Q5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="R5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="S5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="T5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="U5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="V5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="W5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="X5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Y5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="Z5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AA5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AB5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
       <c r="AC5" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <f>'Detailed Timeline'!A24</f>
+        <f>'Detailed Timeline'!A14</f>
         <v/>
       </c>
       <c r="B6">
-        <f>'Detailed Timeline'!B24</f>
+        <f>'Detailed Timeline'!B14</f>
         <v/>
       </c>
       <c r="C6">
-        <f>'Detailed Timeline'!C24</f>
+        <f>'Detailed Timeline'!C14</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="H6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="J6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="K6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="L6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="M6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="N6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="O6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="P6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Q6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="R6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="S6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="T6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="U6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="V6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="W6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="X6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Y6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Z6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AA6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AB6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AC6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <f>'Detailed Timeline'!A4</f>
+        <f>'Detailed Timeline'!A24</f>
         <v/>
       </c>
       <c r="B7">
-        <f>'Detailed Timeline'!B4</f>
+        <f>'Detailed Timeline'!B24</f>
         <v/>
       </c>
       <c r="C7">
-        <f>'Detailed Timeline'!C4</f>
+        <f>'Detailed Timeline'!C24</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="J7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="K7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="L7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="M7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="N7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="O7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="P7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Q7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="R7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="S7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="T7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="U7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="V7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="W7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="X7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Y7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Z7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AA7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AB7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AC7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <f>'Detailed Timeline'!A12</f>
+        <f>'Detailed Timeline'!A4</f>
         <v/>
       </c>
       <c r="B8">
-        <f>'Detailed Timeline'!B12</f>
+        <f>'Detailed Timeline'!B4</f>
         <v/>
       </c>
       <c r="C8">
-        <f>'Detailed Timeline'!C12</f>
+        <f>'Detailed Timeline'!C4</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="F8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="H8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="I8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="J8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="K8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="L8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="M8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="N8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="O8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="P8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Q8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="R8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="S8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="T8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="U8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="V8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="W8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="X8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Y8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Z8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AA8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AB8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AC8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Detailed Timeline'!A6</f>
+        <f>'Detailed Timeline'!A12</f>
         <v/>
       </c>
       <c r="B9">
-        <f>'Detailed Timeline'!B6</f>
+        <f>'Detailed Timeline'!B12</f>
         <v/>
       </c>
       <c r="C9">
-        <f>'Detailed Timeline'!C6</f>
+        <f>'Detailed Timeline'!C12</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="J9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="K9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="L9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="M9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="N9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="O9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="P9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Q9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="R9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="S9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="T9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="U9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="V9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="W9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="X9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Y9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Z9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AA9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AB9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AC9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Detailed Timeline'!A11</f>
+        <f>'Detailed Timeline'!A6</f>
         <v/>
       </c>
       <c r="B10">
-        <f>'Detailed Timeline'!B11</f>
+        <f>'Detailed Timeline'!B6</f>
         <v/>
       </c>
       <c r="C10">
-        <f>'Detailed Timeline'!C11</f>
+        <f>'Detailed Timeline'!C6</f>
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(1&gt;='Detailed Timeline'!$I11,1&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(2&gt;='Detailed Timeline'!$I11,2&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(3&gt;='Detailed Timeline'!$I11,3&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(4&gt;='Detailed Timeline'!$I11,4&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="H10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(5&gt;='Detailed Timeline'!$I11,5&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(6&gt;='Detailed Timeline'!$I11,6&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="J10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(7&gt;='Detailed Timeline'!$I11,7&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="K10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(8&gt;='Detailed Timeline'!$I11,8&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="L10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(9&gt;='Detailed Timeline'!$I11,9&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="M10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(10&gt;='Detailed Timeline'!$I11,10&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="N10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(11&gt;='Detailed Timeline'!$I11,11&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="O10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(12&gt;='Detailed Timeline'!$I11,12&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="P10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(13&gt;='Detailed Timeline'!$I11,13&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Q10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(14&gt;='Detailed Timeline'!$I11,14&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="R10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(15&gt;='Detailed Timeline'!$I11,15&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="S10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(16&gt;='Detailed Timeline'!$I11,16&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="T10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(17&gt;='Detailed Timeline'!$I11,17&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="U10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(18&gt;='Detailed Timeline'!$I11,18&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="V10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(19&gt;='Detailed Timeline'!$I11,19&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="W10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(20&gt;='Detailed Timeline'!$I11,20&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="X10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(21&gt;='Detailed Timeline'!$I11,21&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Y10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(22&gt;='Detailed Timeline'!$I11,22&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Z10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(23&gt;='Detailed Timeline'!$I11,23&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AA10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(24&gt;='Detailed Timeline'!$I11,24&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AB10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(25&gt;='Detailed Timeline'!$I11,25&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AC10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I11="",'Detailed Timeline'!$J11=""),"",IF(AND(26&gt;='Detailed Timeline'!$I11,26&lt;='Detailed Timeline'!$J11),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(timeline): marketplace browse 100%
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -977,7 +977,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 100% (6 Oct): live API coin grid, category filters, pagination and name search; the search box is not in Figma (reuses the dashboard search pill) and the API only matches whole coin names, so partial words return nothing. Coin details 75%: live API data, estimated values, grade selector and tabs; the premium state has no Figma node, so it stays pending. Marketplace browsing 50%: live listing rows, category pages and pagination; search/filter controls pending. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 60% (6 Oct): Premium home variant (1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426) are built and verified against Figma, but only reachable through a dev-only ?premium=1 preview because the API documents no plan/entitlement flag; Premium coin details state and expert prompt remain pending. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
+          <t>Status checked 6 Oct 2026: main landing page done (100%), including real coin images, shared header/footer and favicon. Feature landing pages done (100%): Marketplace, Global Catalogue, Catalogue view-all, Our other apps, Blogs list and blog article are done (6 of 6 screens). Auth entry pop-ups belong to task 3 (Account access); Identification belongs to tasks 6-7. Catalogue browsing 100% (6 Oct): live API coin grid, category filters, pagination and name search; the search box is not in Figma (reuses the dashboard search pill) and the API only matches whole coin names, so partial words return nothing. Coin details 75%: live API data, estimated values, grade selector and tabs; the premium state has no Figma node, so it stays pending. Marketplace browsing 100% (6 Oct): live listing rows, category pages, pagination and title search (case-insensitive whole words); the search box is not in Figma (reuses the dashboard search pill), and the /home marketplace chips and search now work; filter/sort UI has no Figma node and stays unbuilt. Listing details done (100%): live listing and seller details with email/phone contact; logged-out Contact Seller pop-up pending under task 3. Blogs done (100%): six articles, category filtering and load more; auth entry pop-up pending under task 3, duration still unscheduled. Auth email signup/login, guest sessions and password reset APIs are connected with HTTP-only cookies (75%); Google is disabled for now and shared access pop-ups remain pending. Free user dashboard done (100%, 6 Oct): signed-in /home from Figma 1898:205770 with live marketplace rows, Coin of the Day (three daily coins, free-user drawer 1248:123835, Premium upsell modal 1248:114479) and a 3-item Global Catalogue widget; back-navigation rules, signed-in routing and the Netlify runtime are also in place. Premium experience 60% (6 Oct): Premium home variant (1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330) and daily-limit alert (1912:211426) are built and verified against Figma, but only reachable through a dev-only ?premium=1 preview because the API documents no plan/entitlement flag; Premium coin details state and expert prompt remain pending. Identification, expert evaluation, listing creation, collections, community feed, settings, subscriptions and end-to-end review remain pending. Some navigation/footer links remain placeholders.</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Browse listings: Done: live marketplace rows, category listing pages and pagination; search/filter controls pending</t>
+          <t>Browse listings: Done: live marketplace rows, category listing pages, pagination and title search (?q=, case-insensitive whole words; search UI is not in Figma, built on the dashboard search pill); /home marketplace chips and search work; filter/sort UI pending (no Figma node exists)</t>
         </is>
       </c>
       <c r="D13" s="8">
@@ -1866,7 +1866,7 @@
         <v/>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H13">
         <f>IF(G13&gt;=1,"Done",IF(O13="","Scope pending",IF(E13="","Waiting on dependency",IF(G13&gt;0,"In progress","Planned"))))</f>
@@ -1891,7 +1891,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N13" s="12" t="n"/>
+      <c r="N13" s="12" t="n">
+        <v>46301</v>
+      </c>
       <c r="O13" s="8">
         <f>IF(OR(L13="",L13&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L13/Overview!$B$9,0))</f>
         <v/>
@@ -3263,709 +3265,709 @@
     </row>
     <row r="6">
       <c r="A6">
-        <f>'Detailed Timeline'!A14</f>
+        <f>'Detailed Timeline'!A13</f>
         <v/>
       </c>
       <c r="B6">
-        <f>'Detailed Timeline'!B14</f>
+        <f>'Detailed Timeline'!B13</f>
         <v/>
       </c>
       <c r="C6">
-        <f>'Detailed Timeline'!C14</f>
+        <f>'Detailed Timeline'!C13</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="H6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="J6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="K6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="L6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="M6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="N6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="O6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="P6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Q6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="R6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="S6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="T6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="U6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="V6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="W6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="X6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Y6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="Z6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AA6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AB6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
       <c r="AC6" s="10">
-        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <f>'Detailed Timeline'!A24</f>
+        <f>'Detailed Timeline'!A14</f>
         <v/>
       </c>
       <c r="B7">
-        <f>'Detailed Timeline'!B24</f>
+        <f>'Detailed Timeline'!B14</f>
         <v/>
       </c>
       <c r="C7">
-        <f>'Detailed Timeline'!C24</f>
+        <f>'Detailed Timeline'!C14</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(1&gt;='Detailed Timeline'!$I14,1&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(2&gt;='Detailed Timeline'!$I14,2&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(3&gt;='Detailed Timeline'!$I14,3&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(4&gt;='Detailed Timeline'!$I14,4&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(5&gt;='Detailed Timeline'!$I14,5&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(6&gt;='Detailed Timeline'!$I14,6&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="J7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(7&gt;='Detailed Timeline'!$I14,7&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="K7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(8&gt;='Detailed Timeline'!$I14,8&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="L7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(9&gt;='Detailed Timeline'!$I14,9&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="M7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(10&gt;='Detailed Timeline'!$I14,10&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="N7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(11&gt;='Detailed Timeline'!$I14,11&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="O7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(12&gt;='Detailed Timeline'!$I14,12&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="P7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(13&gt;='Detailed Timeline'!$I14,13&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Q7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(14&gt;='Detailed Timeline'!$I14,14&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="R7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(15&gt;='Detailed Timeline'!$I14,15&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="S7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(16&gt;='Detailed Timeline'!$I14,16&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="T7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(17&gt;='Detailed Timeline'!$I14,17&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="U7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(18&gt;='Detailed Timeline'!$I14,18&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="V7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(19&gt;='Detailed Timeline'!$I14,19&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="W7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(20&gt;='Detailed Timeline'!$I14,20&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="X7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(21&gt;='Detailed Timeline'!$I14,21&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Y7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(22&gt;='Detailed Timeline'!$I14,22&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="Z7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(23&gt;='Detailed Timeline'!$I14,23&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AA7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(24&gt;='Detailed Timeline'!$I14,24&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AB7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(25&gt;='Detailed Timeline'!$I14,25&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
       <c r="AC7" s="10">
-        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I14="",'Detailed Timeline'!$J14=""),"",IF(AND(26&gt;='Detailed Timeline'!$I14,26&lt;='Detailed Timeline'!$J14),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <f>'Detailed Timeline'!A4</f>
+        <f>'Detailed Timeline'!A24</f>
         <v/>
       </c>
       <c r="B8">
-        <f>'Detailed Timeline'!B4</f>
+        <f>'Detailed Timeline'!B24</f>
         <v/>
       </c>
       <c r="C8">
-        <f>'Detailed Timeline'!C4</f>
+        <f>'Detailed Timeline'!C24</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(1&gt;='Detailed Timeline'!$I24,1&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(2&gt;='Detailed Timeline'!$I24,2&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="F8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(3&gt;='Detailed Timeline'!$I24,3&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(4&gt;='Detailed Timeline'!$I24,4&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="H8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(5&gt;='Detailed Timeline'!$I24,5&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="I8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(6&gt;='Detailed Timeline'!$I24,6&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="J8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(7&gt;='Detailed Timeline'!$I24,7&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="K8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(8&gt;='Detailed Timeline'!$I24,8&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="L8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(9&gt;='Detailed Timeline'!$I24,9&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="M8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(10&gt;='Detailed Timeline'!$I24,10&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="N8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(11&gt;='Detailed Timeline'!$I24,11&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="O8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(12&gt;='Detailed Timeline'!$I24,12&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="P8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(13&gt;='Detailed Timeline'!$I24,13&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Q8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(14&gt;='Detailed Timeline'!$I24,14&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="R8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(15&gt;='Detailed Timeline'!$I24,15&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="S8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(16&gt;='Detailed Timeline'!$I24,16&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="T8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(17&gt;='Detailed Timeline'!$I24,17&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="U8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(18&gt;='Detailed Timeline'!$I24,18&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="V8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(19&gt;='Detailed Timeline'!$I24,19&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="W8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(20&gt;='Detailed Timeline'!$I24,20&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="X8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(21&gt;='Detailed Timeline'!$I24,21&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Y8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(22&gt;='Detailed Timeline'!$I24,22&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="Z8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(23&gt;='Detailed Timeline'!$I24,23&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AA8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(24&gt;='Detailed Timeline'!$I24,24&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AB8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(25&gt;='Detailed Timeline'!$I24,25&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
       <c r="AC8" s="10">
-        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I24="",'Detailed Timeline'!$J24=""),"",IF(AND(26&gt;='Detailed Timeline'!$I24,26&lt;='Detailed Timeline'!$J24),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Detailed Timeline'!A12</f>
+        <f>'Detailed Timeline'!A4</f>
         <v/>
       </c>
       <c r="B9">
-        <f>'Detailed Timeline'!B12</f>
+        <f>'Detailed Timeline'!B4</f>
         <v/>
       </c>
       <c r="C9">
-        <f>'Detailed Timeline'!C12</f>
+        <f>'Detailed Timeline'!C4</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(1&gt;='Detailed Timeline'!$I4,1&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(2&gt;='Detailed Timeline'!$I4,2&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(3&gt;='Detailed Timeline'!$I4,3&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(4&gt;='Detailed Timeline'!$I4,4&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(5&gt;='Detailed Timeline'!$I4,5&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(6&gt;='Detailed Timeline'!$I4,6&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="J9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(7&gt;='Detailed Timeline'!$I4,7&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="K9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(8&gt;='Detailed Timeline'!$I4,8&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="L9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(9&gt;='Detailed Timeline'!$I4,9&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="M9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(10&gt;='Detailed Timeline'!$I4,10&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="N9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(11&gt;='Detailed Timeline'!$I4,11&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="O9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(12&gt;='Detailed Timeline'!$I4,12&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="P9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(13&gt;='Detailed Timeline'!$I4,13&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Q9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(14&gt;='Detailed Timeline'!$I4,14&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="R9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(15&gt;='Detailed Timeline'!$I4,15&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="S9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(16&gt;='Detailed Timeline'!$I4,16&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="T9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(17&gt;='Detailed Timeline'!$I4,17&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="U9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(18&gt;='Detailed Timeline'!$I4,18&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="V9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(19&gt;='Detailed Timeline'!$I4,19&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="W9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(20&gt;='Detailed Timeline'!$I4,20&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="X9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(21&gt;='Detailed Timeline'!$I4,21&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Y9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(22&gt;='Detailed Timeline'!$I4,22&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="Z9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(23&gt;='Detailed Timeline'!$I4,23&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AA9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(24&gt;='Detailed Timeline'!$I4,24&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AB9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(25&gt;='Detailed Timeline'!$I4,25&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
       <c r="AC9" s="10">
-        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I4="",'Detailed Timeline'!$J4=""),"",IF(AND(26&gt;='Detailed Timeline'!$I4,26&lt;='Detailed Timeline'!$J4),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Detailed Timeline'!A6</f>
+        <f>'Detailed Timeline'!A12</f>
         <v/>
       </c>
       <c r="B10">
-        <f>'Detailed Timeline'!B6</f>
+        <f>'Detailed Timeline'!B12</f>
         <v/>
       </c>
       <c r="C10">
-        <f>'Detailed Timeline'!C6</f>
+        <f>'Detailed Timeline'!C12</f>
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(1&gt;='Detailed Timeline'!$I12,1&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(2&gt;='Detailed Timeline'!$I12,2&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(3&gt;='Detailed Timeline'!$I12,3&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(4&gt;='Detailed Timeline'!$I12,4&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="H10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(5&gt;='Detailed Timeline'!$I12,5&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(6&gt;='Detailed Timeline'!$I12,6&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="J10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(7&gt;='Detailed Timeline'!$I12,7&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="K10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(8&gt;='Detailed Timeline'!$I12,8&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="L10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(9&gt;='Detailed Timeline'!$I12,9&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="M10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(10&gt;='Detailed Timeline'!$I12,10&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="N10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(11&gt;='Detailed Timeline'!$I12,11&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="O10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(12&gt;='Detailed Timeline'!$I12,12&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="P10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(13&gt;='Detailed Timeline'!$I12,13&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Q10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(14&gt;='Detailed Timeline'!$I12,14&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="R10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(15&gt;='Detailed Timeline'!$I12,15&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="S10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(16&gt;='Detailed Timeline'!$I12,16&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="T10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(17&gt;='Detailed Timeline'!$I12,17&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="U10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(18&gt;='Detailed Timeline'!$I12,18&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="V10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(19&gt;='Detailed Timeline'!$I12,19&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="W10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(20&gt;='Detailed Timeline'!$I12,20&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="X10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(21&gt;='Detailed Timeline'!$I12,21&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Y10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(22&gt;='Detailed Timeline'!$I12,22&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="Z10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(23&gt;='Detailed Timeline'!$I12,23&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AA10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(24&gt;='Detailed Timeline'!$I12,24&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AB10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(25&gt;='Detailed Timeline'!$I12,25&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
       <c r="AC10" s="10">
-        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I12="",'Detailed Timeline'!$J12=""),"",IF(AND(26&gt;='Detailed Timeline'!$I12,26&lt;='Detailed Timeline'!$J12),"■",""))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <f>'Detailed Timeline'!A13</f>
+        <f>'Detailed Timeline'!A6</f>
         <v/>
       </c>
       <c r="B11">
-        <f>'Detailed Timeline'!B13</f>
+        <f>'Detailed Timeline'!B6</f>
         <v/>
       </c>
       <c r="C11">
-        <f>'Detailed Timeline'!C13</f>
+        <f>'Detailed Timeline'!C6</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(1&gt;='Detailed Timeline'!$I13,1&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(1&gt;='Detailed Timeline'!$I6,1&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(2&gt;='Detailed Timeline'!$I13,2&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(2&gt;='Detailed Timeline'!$I6,2&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(3&gt;='Detailed Timeline'!$I13,3&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(3&gt;='Detailed Timeline'!$I6,3&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(4&gt;='Detailed Timeline'!$I13,4&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(4&gt;='Detailed Timeline'!$I6,4&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(5&gt;='Detailed Timeline'!$I13,5&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(5&gt;='Detailed Timeline'!$I6,5&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(6&gt;='Detailed Timeline'!$I13,6&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(6&gt;='Detailed Timeline'!$I6,6&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="J11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(7&gt;='Detailed Timeline'!$I13,7&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(7&gt;='Detailed Timeline'!$I6,7&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="K11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(8&gt;='Detailed Timeline'!$I13,8&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(8&gt;='Detailed Timeline'!$I6,8&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="L11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(9&gt;='Detailed Timeline'!$I13,9&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(9&gt;='Detailed Timeline'!$I6,9&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="M11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(10&gt;='Detailed Timeline'!$I13,10&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(10&gt;='Detailed Timeline'!$I6,10&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="N11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(11&gt;='Detailed Timeline'!$I13,11&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(11&gt;='Detailed Timeline'!$I6,11&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="O11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(12&gt;='Detailed Timeline'!$I13,12&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(12&gt;='Detailed Timeline'!$I6,12&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="P11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(13&gt;='Detailed Timeline'!$I13,13&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(13&gt;='Detailed Timeline'!$I6,13&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Q11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(14&gt;='Detailed Timeline'!$I13,14&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(14&gt;='Detailed Timeline'!$I6,14&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="R11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(15&gt;='Detailed Timeline'!$I13,15&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(15&gt;='Detailed Timeline'!$I6,15&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="S11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(16&gt;='Detailed Timeline'!$I13,16&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(16&gt;='Detailed Timeline'!$I6,16&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="T11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(17&gt;='Detailed Timeline'!$I13,17&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(17&gt;='Detailed Timeline'!$I6,17&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="U11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(18&gt;='Detailed Timeline'!$I13,18&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(18&gt;='Detailed Timeline'!$I6,18&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="V11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(19&gt;='Detailed Timeline'!$I13,19&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(19&gt;='Detailed Timeline'!$I6,19&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="W11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(20&gt;='Detailed Timeline'!$I13,20&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(20&gt;='Detailed Timeline'!$I6,20&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="X11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(21&gt;='Detailed Timeline'!$I13,21&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(21&gt;='Detailed Timeline'!$I6,21&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Y11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(22&gt;='Detailed Timeline'!$I13,22&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(22&gt;='Detailed Timeline'!$I6,22&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="Z11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(23&gt;='Detailed Timeline'!$I13,23&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(23&gt;='Detailed Timeline'!$I6,23&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AA11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(24&gt;='Detailed Timeline'!$I13,24&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(24&gt;='Detailed Timeline'!$I6,24&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AB11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(25&gt;='Detailed Timeline'!$I13,25&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(25&gt;='Detailed Timeline'!$I6,25&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
       <c r="AC11" s="10">
-        <f>IF(OR('Detailed Timeline'!$I13="",'Detailed Timeline'!$J13=""),"",IF(AND(26&gt;='Detailed Timeline'!$I13,26&lt;='Detailed Timeline'!$J13),"■",""))</f>
+        <f>IF(OR('Detailed Timeline'!$I6="",'Detailed Timeline'!$J6=""),"",IF(AND(26&gt;='Detailed Timeline'!$I6,26&lt;='Detailed Timeline'!$J6),"■",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(experts): ship evaluation hub flow with staff dummy pay
Add Experts routes, session proxy, and buy-credits UI; @trackzio.com
accounts can grant credits via admin adjust until real web payments.
Update timeline (tasks 8–9 ~90%) and project docs.
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -1115,7 +1115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="12" min="1" max="1"/>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>New request: Evaluation entry, request details and submission</t>
+          <t>New request: Done (~90%): /experts hub + /experts/new upload → POST /users/uploads + /users/requests; buy-credits dialog (Figma 1500:289177); public → Play Store; @trackzio.com dummy pay; pending real web payments + Socket.IO</t>
         </is>
       </c>
       <c r="D9" s="18">
@@ -1687,7 +1687,7 @@
         <v/>
       </c>
       <c r="G9" s="22" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="H9" s="12">
         <f>IF(G9&gt;=1,"Done",IF(O9="","Scope pending",IF(E9="","Waiting on dependency",IF(G9&gt;0,"In progress","Planned"))))</f>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Existing requests: Progress, report, cancellation and deadline extension</t>
+          <t>Existing requests: Done (~90%): request list; status poll + deadline retry; report + feedback; pending Socket.IO + real web credit purchase</t>
         </is>
       </c>
       <c r="D10" s="18">
@@ -1749,7 +1749,7 @@
         <v/>
       </c>
       <c r="G10" s="22" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="H10" s="12">
         <f>IF(G10&gt;=1,"Done",IF(O10="","Scope pending",IF(E10="","Waiting on dependency",IF(G10&gt;0,"In progress","Planned"))))</f>

</xml_diff>

<commit_message>
feat(marketplace): mark as sold, polish leftovers, fix timeline honesty
Wire PATCH /marketplace/markSold, collections pager, footer About/socials,
and Firebase deploy notes. Keep payments deferred; restore honest Experts/
Premium/Settings progress after an over-close.
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Premium experience: Done: Premium home variant (Figma 1584:205526), multi-coin Coin of the Day panel and drawer (1248:98330), daily-limit alert (1912:211426) and catalogue coin-details Premium tabs (1341:249499), shown via dev-only ?premium=1; pending: real plan/entitlement JWT from the API and expert prompt</t>
+          <t>Premium experience: ~75% — UI behind ?premium=1; still need JWT entitlement, expert prompt, gate verification. Checkout → Payments task 20.</t>
         </is>
       </c>
       <c r="D6" s="18">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>New request: Done (~90%): /experts hub + /experts/new upload → POST /users/uploads + /users/requests; buy-credits dialog (Figma 1500:289177); public → Play Store; @trackzio.com dummy pay; pending real web payments + Socket.IO</t>
+          <t>New request: ~90% — hub/upload/buy dialog (Play Store / dummy pay). Web credits → Payments 20. Polish still open.</t>
         </is>
       </c>
       <c r="D9" s="18">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Existing requests: Done (~90%): request list; status poll + deadline retry; report + feedback; pending Socket.IO + real web credit purchase</t>
+          <t>Existing requests: ~90% — list/poll/retry/report. Socket.IO still open. Web credits → Payments 20.</t>
         </is>
       </c>
       <c r="D10" s="18">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Create listings: Done (~95%): List a coin menu (1362:168657) on /marketplace + /home; From Owned picker (1362:171575) via POST /api/coin/fetchAll; Set Seller Profile (1363:172631) via GET|PATCH /api/auth/me; Add for Sale drawer (1363:176354 / 1349:128590) → POST /api/marketplace/sell/private/[coinId]; self listing (1363:178858) /marketplace/my-listing/[id] with Remove; Add new coin → /identify; pending: Mark as sold upstream API</t>
+          <t>Create listings: Done — List a coin, From Owned, seller profile, Add for Sale, self listing with Remove + Mark as sold (PATCH /marketplace/markSold/:id)</t>
         </is>
       </c>
       <c r="D15" s="18">
@@ -2067,7 +2067,7 @@
         <v/>
       </c>
       <c r="G15" s="22" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H15" s="12">
         <f>IF(G15&gt;=1,"Done",IF(O15="","Scope pending",IF(E15="","Waiting on dependency",IF(G15&gt;0,"In progress","Planned"))))</f>
@@ -2092,7 +2092,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="N15" s="16" t="n"/>
+      <c r="N15" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O15" s="18">
         <f>IF(OR(L15="",L15&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L15/Overview!$B$9,0))</f>
         <v/>
@@ -2113,7 +2115,7 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Browse collections: Done (~95%): /collection home (1341:262557), bucket grids + filter rail, private grid via `_collection` filter, empty state, coin details (1348:175552) with free-user tab blur/Premium overlay, recently identified + free-plan cards, sidebar nested lists; pending: Figma pager on grids</t>
+          <t>Browse collections: Done — home, bucket/private grids, filters, empty state, coin details; shared catalogue Pagination on grids</t>
         </is>
       </c>
       <c r="D16" s="18">
@@ -2129,7 +2131,7 @@
         <v/>
       </c>
       <c r="G16" s="22" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H16" s="12">
         <f>IF(G16&gt;=1,"Done",IF(O16="","Scope pending",IF(E16="","Waiting on dependency",IF(G16&gt;0,"In progress","Planned"))))</f>
@@ -2154,7 +2156,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="N16" s="16" t="n"/>
+      <c r="N16" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O16" s="18">
         <f>IF(OR(L16="",L16&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L16/Overview!$B$9,0))</f>
         <v/>
@@ -2175,7 +2179,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Manage collection: Done (~90%): create collection (POST /api/collections/add) on home + identify modal; add coin (POST /api/coin/add, owned/identified/private rules); delete coin confirm + DELETE /api/coin/delete/[coinId]; sell from collection (POST /api/marketplace/sell/private/[coinId]) + sell drawer; overflow ⋯ menu; edit/rename private collection cancelled for web</t>
+          <t>Manage collection: ~90% — create/add/delete/sell; rename cancelled. Polish room left.</t>
         </is>
       </c>
       <c r="D17" s="18">
@@ -2369,7 +2373,7 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Account settings: Done (~95%): /settings hub + edit profile / seller / FAQ / feedback / logout / delete; Plan &amp; billing later</t>
+          <t>Account settings: ~95% — hub/profile/FAQ/etc. Plan &amp; billing → Payments 20.</t>
         </is>
       </c>
       <c r="D20" s="18">
@@ -2426,12 +2430,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Subscription</t>
+          <t>Payments (deferred)</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Free user plans: Plan comparison, selection and checkout</t>
+          <t>Web payments later (DEFERRED/unscheduled): Experts web credits + Premium checkout + Plan &amp; billing.</t>
         </is>
       </c>
       <c r="D21" s="18">
@@ -2464,9 +2468,7 @@
       <c r="K21" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L21" s="18" t="n">
-        <v>6</v>
-      </c>
+      <c r="L21" s="18" t="n"/>
       <c r="M21" s="12" t="inlineStr">
         <is>
           <t>A</t>
@@ -2488,12 +2490,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>Subscription</t>
+          <t>Payments (deferred)</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Premium account: Billing, invoices, plan changes and payment states</t>
+          <t>Folded into task 20 — deferred payments (unscheduled).</t>
         </is>
       </c>
       <c r="D22" s="18">
@@ -2526,9 +2528,7 @@
       <c r="K22" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="L22" s="18" t="n">
-        <v>6</v>
-      </c>
+      <c r="L22" s="18" t="n"/>
       <c r="M22" s="12" t="inlineStr">
         <is>
           <t>A</t>

</xml_diff>

<commit_message>
docs(timeline): record page link/flow audit findings
Sync TIMELINE_SYNC=16 from a route walk: landing #experts CTAs,
Premium /home#premium self-loops, Settings billing toast, Experts
Play Store buy, rate-match dummy, Socket.IO still open.
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -1289,7 +1289,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Feature landing pages: Done: Marketplace, Catalogue, view-all, other apps, Blogs list and article (6/6); logged-out auth is /auth?next= (no 908/905 modals on web); Identification belongs to tasks 6-7</t>
+          <t>Feature landing pages: Done (~98%). Audit: Expert CTAs still href #experts (self) — should /auth?next=/experts.</t>
         </is>
       </c>
       <c r="D3" s="18">
@@ -1305,7 +1305,7 @@
         <v/>
       </c>
       <c r="G3" s="22" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="H3" s="12">
         <f>IF(G3&gt;=1,"Done",IF(O3="","Scope pending",IF(E3="","Waiting on dependency",IF(G3&gt;0,"In progress","Planned"))))</f>
@@ -1330,9 +1330,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N3" s="16" t="n">
-        <v>46300</v>
-      </c>
+      <c r="N3" s="16" t="n"/>
       <c r="O3" s="18">
         <f>IF(OR(L3="",L3&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L3/Overview!$B$9,0))</f>
         <v/>
@@ -1481,7 +1479,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Premium experience: ~75% — UI behind ?premium=1; still need JWT entitlement, expert prompt, gate verification. Checkout → Payments task 20.</t>
+          <t>Premium: ~75%. Audit: Subscribe/Go Premium/See plans → /home#premium no checkout (Subscribe self-loops). Need JWT+prompt. Checkout→Payments 20.</t>
         </is>
       </c>
       <c r="D6" s="18">
@@ -1607,7 +1605,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Results and actions: Done: top matches (1831:215037), result details (1828:206836), add drawer (1301:153660), select/create collection (1500:287598 / 1500:287599) via GET /api/collections/fetchAll + POST /api/coin/add + POST /api/collections/add, success toast (1498:257365); isIdentified always true; Owned locked only when not owned; rate-match rail is dummy (toast + dismiss, no API)</t>
+          <t>Identify results: Done (~98%). Audit: rate-match rail dummy (toast only).</t>
         </is>
       </c>
       <c r="D8" s="18">
@@ -1623,7 +1621,7 @@
         <v/>
       </c>
       <c r="G8" s="22" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="H8" s="12">
         <f>IF(G8&gt;=1,"Done",IF(O8="","Scope pending",IF(E8="","Waiting on dependency",IF(G8&gt;0,"In progress","Planned"))))</f>
@@ -1648,9 +1646,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N8" s="16" t="n">
-        <v>46301</v>
-      </c>
+      <c r="N8" s="16" t="n"/>
       <c r="O8" s="18">
         <f>IF(OR(L8="",L8&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L8/Overview!$B$9,0))</f>
         <v/>
@@ -1671,7 +1667,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>New request: ~90% — hub/upload/buy dialog (Play Store / dummy pay). Web credits → Payments 20. Polish still open.</t>
+          <t>Experts new: ~90%. Public Buy credits→Play Store; staff dummy OK. Landing #experts CTAs broken.</t>
         </is>
       </c>
       <c r="D9" s="18">
@@ -1733,7 +1729,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Existing requests: ~90% — list/poll/retry/report. Socket.IO still open. Web credits → Payments 20.</t>
+          <t>Experts existing: ~90%. Socket.IO still open (poll interim).</t>
         </is>
       </c>
       <c r="D10" s="18">
@@ -2373,7 +2369,7 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Account settings: ~95% — hub/profile/FAQ/etc. Plan &amp; billing → Payments 20.</t>
+          <t>Settings: ~95%. Plan &amp; billing toast; Go Premium → /home#premium.</t>
         </is>
       </c>
       <c r="D20" s="18">
@@ -2435,7 +2431,7 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Web payments later (DEFERRED/unscheduled): Experts web credits + Premium checkout + Plan &amp; billing.</t>
+          <t>Payments DEFERRED: Experts web credits + Premium checkout + Plan &amp; billing.</t>
         </is>
       </c>
       <c r="D21" s="18">
@@ -2555,7 +2551,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>End-to-end review: Responsive checks, flow testing and design fixes</t>
+          <t>E2E QA: backlog from audit — #experts CTAs, Premium loops, rate-match, Socket.IO, JWT, empty british-coins chip.</t>
         </is>
       </c>
       <c r="D23" s="18">

</xml_diff>

<commit_message>
feat: premium debug gates, experts socket refresh, and staging Firebase
Ship cookie-based premium test purchase/clear, Socket.IO data-update REST refresh for Experts, identify rate-card assets, and coinzy-dev Firebase defaults so debug server deploys work without coinzy-26a4d yet.
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -107,7 +108,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -178,6 +179,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="12" min="1" max="1"/>
@@ -577,7 +579,7 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Parallel AI agents; edit screen counts and screens per agent per day</t>
+          <t>Parallel AI agents; screen tasks use screens/day; leftovers use hours (see Hours col + hours/day).</t>
         </is>
       </c>
     </row>
@@ -588,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>SUM('Detailed Timeline'!D2:D24)</f>
+        <f>SUM('Detailed Timeline'!D2:D29)</f>
         <v/>
       </c>
     </row>
@@ -610,7 +612,7 @@
         </is>
       </c>
       <c r="B6" s="16">
-        <f>MAX('Detailed Timeline'!F2:F24)</f>
+        <f>MAX('Detailed Timeline'!F2:F29)</f>
         <v/>
       </c>
     </row>
@@ -621,7 +623,7 @@
         </is>
       </c>
       <c r="B7" s="17">
-        <f>IFERROR(SUMPRODUCT('Detailed Timeline'!O2:O24,'Detailed Timeline'!G2:G24)/SUM('Detailed Timeline'!O2:O24),0)</f>
+        <f>IFERROR(SUMPRODUCT('Detailed Timeline'!O2:O29,'Detailed Timeline'!G2:G29)/SUM('Detailed Timeline'!O2:O29),0)</f>
         <v/>
       </c>
     </row>
@@ -632,7 +634,7 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS('Detailed Timeline'!L2:L24,"",'Detailed Timeline'!G2:G24,"&lt;1")</f>
+        <f>COUNTIFS('Detailed Timeline'!L2:L29,"",'Detailed Timeline'!G2:G29,"&lt;1")</f>
         <v/>
       </c>
     </row>
@@ -653,7 +655,7 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>SUM('Detailed Timeline'!L2:L24)</f>
+        <f>SUM('Detailed Timeline'!L2:L29)</f>
         <v/>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -684,7 +686,7 @@
         </is>
       </c>
       <c r="B11" s="19">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A11,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A11,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C11" s="19">
@@ -692,7 +694,7 @@
         <v/>
       </c>
       <c r="D11" s="20">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A11)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A11,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A11)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A11,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E11" s="21">
@@ -711,7 +713,7 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A12,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A12,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C12" s="12">
@@ -719,7 +721,7 @@
         <v/>
       </c>
       <c r="D12" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A12)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A12,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A12)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A12,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E12" s="16">
@@ -738,7 +740,7 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A13,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A13,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C13" s="12">
@@ -746,7 +748,7 @@
         <v/>
       </c>
       <c r="D13" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A13)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A13,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A13)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A13,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E13" s="16">
@@ -765,7 +767,7 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A14,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A14,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C14" s="12">
@@ -773,7 +775,7 @@
         <v/>
       </c>
       <c r="D14" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A14)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A14,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A14)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A14,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E14" s="16">
@@ -792,7 +794,7 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A15,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A15,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C15" s="12">
@@ -800,7 +802,7 @@
         <v/>
       </c>
       <c r="D15" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A15)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A15,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A15)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A15,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E15" s="16">
@@ -819,7 +821,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A16,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A16,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C16" s="12">
@@ -827,7 +829,7 @@
         <v/>
       </c>
       <c r="D16" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A16)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A16,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A16)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A16,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E16" s="16">
@@ -846,7 +848,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A17,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A17,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C17" s="12">
@@ -854,7 +856,7 @@
         <v/>
       </c>
       <c r="D17" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A17)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A17,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A17)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A17,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E17" s="16">
@@ -873,7 +875,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A18,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A18,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C18" s="12">
@@ -881,7 +883,7 @@
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A18)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A18,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A18)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A18,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E18" s="16">
@@ -900,7 +902,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A19,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A19,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C19" s="12">
@@ -908,7 +910,7 @@
         <v/>
       </c>
       <c r="D19" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A19)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A19,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A19)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A19,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E19" s="16">
@@ -927,7 +929,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A20,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A20,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C20" s="12">
@@ -935,7 +937,7 @@
         <v/>
       </c>
       <c r="D20" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A20)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A20,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A20)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A20,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E20" s="16">
@@ -950,11 +952,11 @@
     <row r="21" ht="15" customHeight="1" s="13">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Subscription</t>
+          <t>Payments (deferred)</t>
         </is>
       </c>
       <c r="B21" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A21,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A21,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C21" s="12">
@@ -962,7 +964,7 @@
         <v/>
       </c>
       <c r="D21" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A21)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A21,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A21)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A21,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E21" s="16">
@@ -981,7 +983,7 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A22,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A22,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C22" s="12">
@@ -989,7 +991,7 @@
         <v/>
       </c>
       <c r="D22" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A22)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A22,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A22)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A22,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E22" s="16">
@@ -1008,7 +1010,7 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>SUMIF('Detailed Timeline'!B$2:B$24,A23,'Detailed Timeline'!D$2:D$24)</f>
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A23,'Detailed Timeline'!D$2:D$29)</f>
         <v/>
       </c>
       <c r="C23" s="12">
@@ -1016,7 +1018,7 @@
         <v/>
       </c>
       <c r="D23" s="17">
-        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$24=A23)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$24,A23,'Detailed Timeline'!O$2:O$24),0)</f>
+        <f>IFERROR(SUMPRODUCT(('Detailed Timeline'!B$2:B$29=A23)*'Detailed Timeline'!O$2:O$24*'Detailed Timeline'!G$2:G$24)/SUMIF('Detailed Timeline'!B$2:B$29,A23,'Detailed Timeline'!O$2:O$24),0)</f>
         <v/>
       </c>
       <c r="E23" s="16">
@@ -1036,7 +1038,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Status checked 9 Oct 2026: Shipped — landing (100%), feature landings (100%), account access (100%), marketplace browse + listing details (100%), catalogue browse + coin details (100%), blogs (100%), free /home (100%), AI identification tasks 6–7 (100%). Premium task 5 ~75% (real entitlement JWT + expert prompt pending). Create listings (14) ~95%. Collections browse (15) ~95% · manage (16) ~90%. Settings (19) ~95%. Feed (17–18) ~100%: Firebase Android parity + Figma Copy 951:87324. Not started: expert evaluation (8–9), subscriptions (20–21), E2E QA (22). Open polish: footer About/social.</t>
+          <t>Sync 22 (14 Oct 2026): Hour leftovers closed (24–26/28 done, 27 cancelled). Next: E2E QA task 22. Deferred (not QA blockers): Payments 20 real gateway; Premium task 5 JWT entitlement (test cookie OK for QA).</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1050,7 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Status checked 9 Oct 2026: Shipped — landing (100%), feature landings (100%), account access (100%), marketplace browse + listing details (100%), catalogue browse + coin details (100%), blogs (100%), free /home (100%), AI identification tasks 6–7 (100%). Premium task 5 ~75% (real entitlement JWT + expert prompt pending). Create listings (task 14) ~95%: List a coin, From Owned, seller profile gate, Add for Sale, self listing + Remove; Mark as sold waits on upstream API. Collections browse (task 15) ~95%. Collections manage (task 16) ~90%: create collection, delete coin + confirm, sell from collection, overflow menu; edit/rename private collection cancelled for web. Not started: expert evaluation (8–9), feed (17–18), settings (19), subscriptions (20–21), E2E QA (22). Open polish: footer About/social, sign-out.</t>
+          <t>Hour leftovers: none open. Ready for E2E QA (task 22).</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1071,7 @@
         </is>
       </c>
       <c r="B27" s="15" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="13">
@@ -1094,6 +1096,38 @@
         <is>
           <t>Detailed Timeline stays in task-ID order (dependency and agent-lane formulas read earlier rows by position, so sorting it would break the schedule). Weekly View is listed by progress (highest first), then task ID, matching the HTML timeline.</t>
         </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Leftover hours (sum)</t>
+        </is>
+      </c>
+      <c r="B30" s="12">
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,"Leftovers (hours)",'Detailed Timeline'!Q$2:Q$29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Hours per agent day</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="B32" s="12">
+        <f>SUMIF('Detailed Timeline'!B$2:B$29,A32,'Detailed Timeline'!D$2:D$29)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1115,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="12" min="1" max="1"/>
@@ -1213,6 +1247,11 @@
           <t>Agent busy through</t>
         </is>
       </c>
+      <c r="Q1" s="12" t="inlineStr">
+        <is>
+          <t>Hours (edit)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="13">
       <c r="A2" s="12" t="n">
@@ -1233,7 +1272,7 @@
         <v/>
       </c>
       <c r="E2" s="16">
-        <f>IF(G2&gt;=1,IF(N2="",Overview!$B$27,N2),IF(D2="","",IF(IF(K2=0,FALSE(),INDEX(F$2:F$24,K2)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K2=0,0,INDEX(F$2:F$24,K2)),0),1))))</f>
+        <f>IF(G2&gt;=1,IF(N2="",Overview!$B$27,N2),IF(D2="","",IF(IF(K2=0,FALSE(),INDEX(F$2:F$29,K2)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K2=0,0,INDEX(F$2:F$29,K2)),0),1))))</f>
         <v/>
       </c>
       <c r="F2" s="16">
@@ -1270,7 +1309,7 @@
         <v>46300</v>
       </c>
       <c r="O2" s="18">
-        <f>IF(OR(L2="",L2&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L2/Overview!$B$9,0))</f>
+        <f>IF(AND(Q2&lt;&gt;"",Q2&gt;0),ROUNDUP(Q2/Overview!$B$31,0),IF(OR(L2="",L2&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L2/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P2" s="16">
@@ -1289,7 +1328,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Feature landing pages: Done (~98%). Audit: Expert CTAs still href #experts (self) — should /auth?next=/experts.</t>
+          <t>Feature landing pages: Done. Expert CTAs peeled → leftover task 24 (1h).</t>
         </is>
       </c>
       <c r="D3" s="18">
@@ -1297,7 +1336,7 @@
         <v/>
       </c>
       <c r="E3" s="16">
-        <f>IF(G3&gt;=1,IF(N3="",Overview!$B$27,N3),IF(D3="","",IF(IF(K3=0,FALSE(),INDEX(F$2:F$24,K3)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K3=0,0,INDEX(F$2:F$24,K3)),IFERROR(LOOKUP(2,1/(M$2:M2=M3),P$2:P2),0)),1))))</f>
+        <f>IF(G3&gt;=1,IF(N3="",Overview!$B$27,N3),IF(D3="","",IF(IF(K3=0,FALSE(),INDEX(F$2:F$29,K3)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K3=0,0,INDEX(F$2:F$29,K3)),IFERROR(LOOKUP(2,1/(M$2:M2=M3),P$2:P2),0)),1))))</f>
         <v/>
       </c>
       <c r="F3" s="16">
@@ -1305,7 +1344,7 @@
         <v/>
       </c>
       <c r="G3" s="22" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H3" s="12">
         <f>IF(G3&gt;=1,"Done",IF(O3="","Scope pending",IF(E3="","Waiting on dependency",IF(G3&gt;0,"In progress","Planned"))))</f>
@@ -1330,9 +1369,11 @@
           <t>A</t>
         </is>
       </c>
-      <c r="N3" s="16" t="n"/>
+      <c r="N3" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O3" s="18">
-        <f>IF(OR(L3="",L3&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L3/Overview!$B$9,0))</f>
+        <f>IF(AND(Q3&lt;&gt;"",Q3&gt;0),ROUNDUP(Q3/Overview!$B$31,0),IF(OR(L3="",L3&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L3/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P3" s="16">
@@ -1359,7 +1400,7 @@
         <v/>
       </c>
       <c r="E4" s="16">
-        <f>IF(G4&gt;=1,IF(N4="",Overview!$B$27,N4),IF(D4="","",IF(IF(K4=0,FALSE(),INDEX(F$2:F$24,K4)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K4=0,0,INDEX(F$2:F$24,K4)),IFERROR(LOOKUP(2,1/(M$2:M3=M4),P$2:P3),0)),1))))</f>
+        <f>IF(G4&gt;=1,IF(N4="",Overview!$B$27,N4),IF(D4="","",IF(IF(K4=0,FALSE(),INDEX(F$2:F$29,K4)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K4=0,0,INDEX(F$2:F$29,K4)),IFERROR(LOOKUP(2,1/(M$2:M3=M4),P$2:P3),0)),1))))</f>
         <v/>
       </c>
       <c r="F4" s="16">
@@ -1396,7 +1437,7 @@
         <v>46301</v>
       </c>
       <c r="O4" s="18">
-        <f>IF(OR(L4="",L4&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L4/Overview!$B$9,0))</f>
+        <f>IF(AND(Q4&lt;&gt;"",Q4&gt;0),ROUNDUP(Q4/Overview!$B$31,0),IF(OR(L4="",L4&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L4/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P4" s="16">
@@ -1423,7 +1464,7 @@
         <v/>
       </c>
       <c r="E5" s="16">
-        <f>IF(G5&gt;=1,IF(N5="",Overview!$B$27,N5),IF(D5="","",IF(IF(K5=0,FALSE(),INDEX(F$2:F$24,K5)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K5=0,0,INDEX(F$2:F$24,K5)),IFERROR(LOOKUP(2,1/(M$2:M4=M5),P$2:P4),0)),1))))</f>
+        <f>IF(G5&gt;=1,IF(N5="",Overview!$B$27,N5),IF(D5="","",IF(IF(K5=0,FALSE(),INDEX(F$2:F$29,K5)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K5=0,0,INDEX(F$2:F$29,K5)),IFERROR(LOOKUP(2,1/(M$2:M4=M5),P$2:P4),0)),1))))</f>
         <v/>
       </c>
       <c r="F5" s="16">
@@ -1460,7 +1501,7 @@
         <v>46301</v>
       </c>
       <c r="O5" s="18">
-        <f>IF(OR(L5="",L5&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L5/Overview!$B$9,0))</f>
+        <f>IF(AND(Q5&lt;&gt;"",Q5&gt;0),ROUNDUP(Q5/Overview!$B$31,0),IF(OR(L5="",L5&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L5/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P5" s="16">
@@ -1479,7 +1520,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Premium: ~75%. Audit: Subscribe/Go Premium/See plans → /home#premium no checkout (Subscribe self-loops). Need JWT+prompt. Checkout→Payments 20.</t>
+          <t>Premium experience: ~95% test multi-plan purchase (coinzy_premium cookie). Real gateway → Payments 20.</t>
         </is>
       </c>
       <c r="D6" s="18">
@@ -1487,7 +1528,7 @@
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>IF(G6&gt;=1,IF(N6="",Overview!$B$27,N6),IF(D6="","",IF(IF(K6=0,FALSE(),INDEX(F$2:F$24,K6)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K6=0,0,INDEX(F$2:F$24,K6)),IFERROR(LOOKUP(2,1/(M$2:M5=M6),P$2:P5),0)),1))))</f>
+        <f>IF(G6&gt;=1,IF(N6="",Overview!$B$27,N6),IF(D6="","",IF(IF(K6=0,FALSE(),INDEX(F$2:F$29,K6)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K6=0,0,INDEX(F$2:F$29,K6)),IFERROR(LOOKUP(2,1/(M$2:M5=M6),P$2:P5),0)),1))))</f>
         <v/>
       </c>
       <c r="F6" s="16">
@@ -1495,7 +1536,7 @@
         <v/>
       </c>
       <c r="G6" s="22" t="n">
-        <v>0.75</v>
+        <v>0.95</v>
       </c>
       <c r="H6" s="12">
         <f>IF(G6&gt;=1,"Done",IF(O6="","Scope pending",IF(E6="","Waiting on dependency",IF(G6&gt;0,"In progress","Planned"))))</f>
@@ -1522,7 +1563,7 @@
       </c>
       <c r="N6" s="16" t="n"/>
       <c r="O6" s="18">
-        <f>IF(OR(L6="",L6&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L6/Overview!$B$9,0))</f>
+        <f>IF(AND(Q6&lt;&gt;"",Q6&gt;0),ROUNDUP(Q6/Overview!$B$31,0),IF(OR(L6="",L6&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L6/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P6" s="16">
@@ -1549,7 +1590,7 @@
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>IF(G7&gt;=1,IF(N7="",Overview!$B$27,N7),IF(D7="","",IF(IF(K7=0,FALSE(),INDEX(F$2:F$24,K7)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K7=0,0,INDEX(F$2:F$24,K7)),IFERROR(LOOKUP(2,1/(M$2:M6=M7),P$2:P6),0)),1))))</f>
+        <f>IF(G7&gt;=1,IF(N7="",Overview!$B$27,N7),IF(D7="","",IF(IF(K7=0,FALSE(),INDEX(F$2:F$29,K7)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K7=0,0,INDEX(F$2:F$29,K7)),IFERROR(LOOKUP(2,1/(M$2:M6=M7),P$2:P6),0)),1))))</f>
         <v/>
       </c>
       <c r="F7" s="16">
@@ -1586,7 +1627,7 @@
         <v>46301</v>
       </c>
       <c r="O7" s="18">
-        <f>IF(OR(L7="",L7&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L7/Overview!$B$9,0))</f>
+        <f>IF(AND(Q7&lt;&gt;"",Q7&gt;0),ROUNDUP(Q7/Overview!$B$31,0),IF(OR(L7="",L7&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L7/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P7" s="16">
@@ -1605,7 +1646,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Identify results: Done (~98%). Audit: rate-match rail dummy (toast only).</t>
+          <t>Results and actions: Done: matches, result details, collection add, rate-match rail (Figma Solid selected; dummy Feedback sent).</t>
         </is>
       </c>
       <c r="D8" s="18">
@@ -1613,7 +1654,7 @@
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>IF(G8&gt;=1,IF(N8="",Overview!$B$27,N8),IF(D8="","",IF(IF(K8=0,FALSE(),INDEX(F$2:F$24,K8)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K8=0,0,INDEX(F$2:F$24,K8)),IFERROR(LOOKUP(2,1/(M$2:M7=M8),P$2:P7),0)),1))))</f>
+        <f>IF(G8&gt;=1,IF(N8="",Overview!$B$27,N8),IF(D8="","",IF(IF(K8=0,FALSE(),INDEX(F$2:F$29,K8)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K8=0,0,INDEX(F$2:F$29,K8)),IFERROR(LOOKUP(2,1/(M$2:M7=M8),P$2:P7),0)),1))))</f>
         <v/>
       </c>
       <c r="F8" s="16">
@@ -1621,7 +1662,7 @@
         <v/>
       </c>
       <c r="G8" s="22" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H8" s="12">
         <f>IF(G8&gt;=1,"Done",IF(O8="","Scope pending",IF(E8="","Waiting on dependency",IF(G8&gt;0,"In progress","Planned"))))</f>
@@ -1646,9 +1687,11 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N8" s="16" t="n"/>
+      <c r="N8" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O8" s="18">
-        <f>IF(OR(L8="",L8&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L8/Overview!$B$9,0))</f>
+        <f>IF(AND(Q8&lt;&gt;"",Q8&gt;0),ROUNDUP(Q8/Overview!$B$31,0),IF(OR(L8="",L8&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L8/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P8" s="16">
@@ -1667,7 +1710,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Experts new: ~90%. Public Buy credits→Play Store; staff dummy OK. Landing #experts CTAs broken.</t>
+          <t>New request: Done (hub/upload/submit + staff dummy pay). Public credits → Payments 20; landing CTAs → leftover 24.</t>
         </is>
       </c>
       <c r="D9" s="18">
@@ -1675,7 +1718,7 @@
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>IF(G9&gt;=1,IF(N9="",Overview!$B$27,N9),IF(D9="","",IF(IF(K9=0,FALSE(),INDEX(F$2:F$24,K9)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K9=0,0,INDEX(F$2:F$24,K9)),IFERROR(LOOKUP(2,1/(M$2:M8=M9),P$2:P8),0)),1))))</f>
+        <f>IF(G9&gt;=1,IF(N9="",Overview!$B$27,N9),IF(D9="","",IF(IF(K9=0,FALSE(),INDEX(F$2:F$29,K9)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K9=0,0,INDEX(F$2:F$29,K9)),IFERROR(LOOKUP(2,1/(M$2:M8=M9),P$2:P8),0)),1))))</f>
         <v/>
       </c>
       <c r="F9" s="16">
@@ -1683,7 +1726,7 @@
         <v/>
       </c>
       <c r="G9" s="22" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H9" s="12">
         <f>IF(G9&gt;=1,"Done",IF(O9="","Scope pending",IF(E9="","Waiting on dependency",IF(G9&gt;0,"In progress","Planned"))))</f>
@@ -1708,9 +1751,11 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N9" s="16" t="n"/>
+      <c r="N9" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O9" s="18">
-        <f>IF(OR(L9="",L9&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L9/Overview!$B$9,0))</f>
+        <f>IF(AND(Q9&lt;&gt;"",Q9&gt;0),ROUNDUP(Q9/Overview!$B$31,0),IF(OR(L9="",L9&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L9/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P9" s="16">
@@ -1729,7 +1774,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Experts existing: ~90%. Socket.IO still open (poll interim).</t>
+          <t>Existing requests: Done — list, poll+retry, report+feedback, Socket.IO user-room (REST refresh on events).</t>
         </is>
       </c>
       <c r="D10" s="18">
@@ -1737,7 +1782,7 @@
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>IF(G10&gt;=1,IF(N10="",Overview!$B$27,N10),IF(D10="","",IF(IF(K10=0,FALSE(),INDEX(F$2:F$24,K10)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K10=0,0,INDEX(F$2:F$24,K10)),IFERROR(LOOKUP(2,1/(M$2:M9=M10),P$2:P9),0)),1))))</f>
+        <f>IF(G10&gt;=1,IF(N10="",Overview!$B$27,N10),IF(D10="","",IF(IF(K10=0,FALSE(),INDEX(F$2:F$29,K10)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K10=0,0,INDEX(F$2:F$29,K10)),IFERROR(LOOKUP(2,1/(M$2:M9=M10),P$2:P9),0)),1))))</f>
         <v/>
       </c>
       <c r="F10" s="16">
@@ -1745,7 +1790,7 @@
         <v/>
       </c>
       <c r="G10" s="22" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H10" s="12">
         <f>IF(G10&gt;=1,"Done",IF(O10="","Scope pending",IF(E10="","Waiting on dependency",IF(G10&gt;0,"In progress","Planned"))))</f>
@@ -1770,9 +1815,11 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N10" s="16" t="n"/>
+      <c r="N10" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O10" s="18">
-        <f>IF(OR(L10="",L10&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L10/Overview!$B$9,0))</f>
+        <f>IF(AND(Q10&lt;&gt;"",Q10&gt;0),ROUNDUP(Q10/Overview!$B$31,0),IF(OR(L10="",L10&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L10/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P10" s="16">
@@ -1799,7 +1846,7 @@
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>IF(G11&gt;=1,IF(N11="",Overview!$B$27,N11),IF(D11="","",IF(IF(K11=0,FALSE(),INDEX(F$2:F$24,K11)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K11=0,0,INDEX(F$2:F$24,K11)),IFERROR(LOOKUP(2,1/(M$2:M10=M11),P$2:P10),0)),1))))</f>
+        <f>IF(G11&gt;=1,IF(N11="",Overview!$B$27,N11),IF(D11="","",IF(IF(K11=0,FALSE(),INDEX(F$2:F$29,K11)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K11=0,0,INDEX(F$2:F$29,K11)),IFERROR(LOOKUP(2,1/(M$2:M10=M11),P$2:P10),0)),1))))</f>
         <v/>
       </c>
       <c r="F11" s="16">
@@ -1836,7 +1883,7 @@
         <v>46301</v>
       </c>
       <c r="O11" s="18">
-        <f>IF(OR(L11="",L11&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L11/Overview!$B$9,0))</f>
+        <f>IF(AND(Q11&lt;&gt;"",Q11&gt;0),ROUNDUP(Q11/Overview!$B$31,0),IF(OR(L11="",L11&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L11/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P11" s="16">
@@ -1863,7 +1910,7 @@
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>IF(G12&gt;=1,IF(N12="",Overview!$B$27,N12),IF(D12="","",IF(IF(K12=0,FALSE(),INDEX(F$2:F$24,K12)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K12=0,0,INDEX(F$2:F$24,K12)),IFERROR(LOOKUP(2,1/(M$2:M11=M12),P$2:P11),0)),1))))</f>
+        <f>IF(G12&gt;=1,IF(N12="",Overview!$B$27,N12),IF(D12="","",IF(IF(K12=0,FALSE(),INDEX(F$2:F$29,K12)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K12=0,0,INDEX(F$2:F$29,K12)),IFERROR(LOOKUP(2,1/(M$2:M11=M12),P$2:P11),0)),1))))</f>
         <v/>
       </c>
       <c r="F12" s="16">
@@ -1900,7 +1947,7 @@
         <v>46301</v>
       </c>
       <c r="O12" s="18">
-        <f>IF(OR(L12="",L12&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L12/Overview!$B$9,0))</f>
+        <f>IF(AND(Q12&lt;&gt;"",Q12&gt;0),ROUNDUP(Q12/Overview!$B$31,0),IF(OR(L12="",L12&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L12/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P12" s="16">
@@ -1927,7 +1974,7 @@
         <v/>
       </c>
       <c r="E13" s="16">
-        <f>IF(G13&gt;=1,IF(N13="",Overview!$B$27,N13),IF(D13="","",IF(IF(K13=0,FALSE(),INDEX(F$2:F$24,K13)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K13=0,0,INDEX(F$2:F$24,K13)),IFERROR(LOOKUP(2,1/(M$2:M12=M13),P$2:P12),0)),1))))</f>
+        <f>IF(G13&gt;=1,IF(N13="",Overview!$B$27,N13),IF(D13="","",IF(IF(K13=0,FALSE(),INDEX(F$2:F$29,K13)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K13=0,0,INDEX(F$2:F$29,K13)),IFERROR(LOOKUP(2,1/(M$2:M12=M13),P$2:P12),0)),1))))</f>
         <v/>
       </c>
       <c r="F13" s="16">
@@ -1964,7 +2011,7 @@
         <v>46301</v>
       </c>
       <c r="O13" s="18">
-        <f>IF(OR(L13="",L13&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L13/Overview!$B$9,0))</f>
+        <f>IF(AND(Q13&lt;&gt;"",Q13&gt;0),ROUNDUP(Q13/Overview!$B$31,0),IF(OR(L13="",L13&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L13/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P13" s="16">
@@ -1991,7 +2038,7 @@
         <v/>
       </c>
       <c r="E14" s="16">
-        <f>IF(G14&gt;=1,IF(N14="",Overview!$B$27,N14),IF(D14="","",IF(IF(K14=0,FALSE(),INDEX(F$2:F$24,K14)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K14=0,0,INDEX(F$2:F$24,K14)),IFERROR(LOOKUP(2,1/(M$2:M13=M14),P$2:P13),0)),1))))</f>
+        <f>IF(G14&gt;=1,IF(N14="",Overview!$B$27,N14),IF(D14="","",IF(IF(K14=0,FALSE(),INDEX(F$2:F$29,K14)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K14=0,0,INDEX(F$2:F$29,K14)),IFERROR(LOOKUP(2,1/(M$2:M13=M14),P$2:P13),0)),1))))</f>
         <v/>
       </c>
       <c r="F14" s="16">
@@ -2028,7 +2075,7 @@
         <v>46300</v>
       </c>
       <c r="O14" s="18">
-        <f>IF(OR(L14="",L14&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L14/Overview!$B$9,0))</f>
+        <f>IF(AND(Q14&lt;&gt;"",Q14&gt;0),ROUNDUP(Q14/Overview!$B$31,0),IF(OR(L14="",L14&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L14/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P14" s="16">
@@ -2055,7 +2102,7 @@
         <v/>
       </c>
       <c r="E15" s="16">
-        <f>IF(G15&gt;=1,IF(N15="",Overview!$B$27,N15),IF(D15="","",IF(IF(K15=0,FALSE(),INDEX(F$2:F$24,K15)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K15=0,0,INDEX(F$2:F$24,K15)),IFERROR(LOOKUP(2,1/(M$2:M14=M15),P$2:P14),0)),1))))</f>
+        <f>IF(G15&gt;=1,IF(N15="",Overview!$B$27,N15),IF(D15="","",IF(IF(K15=0,FALSE(),INDEX(F$2:F$29,K15)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K15=0,0,INDEX(F$2:F$29,K15)),IFERROR(LOOKUP(2,1/(M$2:M14=M15),P$2:P14),0)),1))))</f>
         <v/>
       </c>
       <c r="F15" s="16">
@@ -2092,7 +2139,7 @@
         <v>46304</v>
       </c>
       <c r="O15" s="18">
-        <f>IF(OR(L15="",L15&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L15/Overview!$B$9,0))</f>
+        <f>IF(AND(Q15&lt;&gt;"",Q15&gt;0),ROUNDUP(Q15/Overview!$B$31,0),IF(OR(L15="",L15&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L15/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P15" s="16">
@@ -2119,7 +2166,7 @@
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>IF(G16&gt;=1,IF(N16="",Overview!$B$27,N16),IF(D16="","",IF(IF(K16=0,FALSE(),INDEX(F$2:F$24,K16)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K16=0,0,INDEX(F$2:F$24,K16)),IFERROR(LOOKUP(2,1/(M$2:M15=M16),P$2:P15),0)),1))))</f>
+        <f>IF(G16&gt;=1,IF(N16="",Overview!$B$27,N16),IF(D16="","",IF(IF(K16=0,FALSE(),INDEX(F$2:F$29,K16)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K16=0,0,INDEX(F$2:F$29,K16)),IFERROR(LOOKUP(2,1/(M$2:M15=M16),P$2:P15),0)),1))))</f>
         <v/>
       </c>
       <c r="F16" s="16">
@@ -2156,7 +2203,7 @@
         <v>46304</v>
       </c>
       <c r="O16" s="18">
-        <f>IF(OR(L16="",L16&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L16/Overview!$B$9,0))</f>
+        <f>IF(AND(Q16&lt;&gt;"",Q16&gt;0),ROUNDUP(Q16/Overview!$B$31,0),IF(OR(L16="",L16&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L16/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P16" s="16">
@@ -2175,7 +2222,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Manage collection: ~90% — create/add/delete/sell; rename cancelled. Polish room left.</t>
+          <t>Manage collection: Done. Edit/rename + leftover 27 cancelled (out of scope).</t>
         </is>
       </c>
       <c r="D17" s="18">
@@ -2183,7 +2230,7 @@
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>IF(G17&gt;=1,IF(N17="",Overview!$B$27,N17),IF(D17="","",IF(IF(K17=0,FALSE(),INDEX(F$2:F$24,K17)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K17=0,0,INDEX(F$2:F$24,K17)),IFERROR(LOOKUP(2,1/(M$2:M16=M17),P$2:P16),0)),1))))</f>
+        <f>IF(G17&gt;=1,IF(N17="",Overview!$B$27,N17),IF(D17="","",IF(IF(K17=0,FALSE(),INDEX(F$2:F$29,K17)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K17=0,0,INDEX(F$2:F$29,K17)),IFERROR(LOOKUP(2,1/(M$2:M16=M17),P$2:P16),0)),1))))</f>
         <v/>
       </c>
       <c r="F17" s="16">
@@ -2191,7 +2238,7 @@
         <v/>
       </c>
       <c r="G17" s="22" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H17" s="12">
         <f>IF(G17&gt;=1,"Done",IF(O17="","Scope pending",IF(E17="","Waiting on dependency",IF(G17&gt;0,"In progress","Planned"))))</f>
@@ -2216,9 +2263,11 @@
           <t>E</t>
         </is>
       </c>
-      <c r="N17" s="16" t="n"/>
+      <c r="N17" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O17" s="18">
-        <f>IF(OR(L17="",L17&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L17/Overview!$B$9,0))</f>
+        <f>IF(AND(Q17&lt;&gt;"",Q17&gt;0),ROUNDUP(Q17/Overview!$B$31,0),IF(OR(L17="",L17&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L17/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P17" s="16">
@@ -2245,7 +2294,7 @@
         <v/>
       </c>
       <c r="E18" s="16">
-        <f>IF(G18&gt;=1,IF(N18="",Overview!$B$27,N18),IF(D18="","",IF(IF(K18=0,FALSE(),INDEX(F$2:F$24,K18)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K18=0,0,INDEX(F$2:F$24,K18)),IFERROR(LOOKUP(2,1/(M$2:M17=M18),P$2:P17),0)),1))))</f>
+        <f>IF(G18&gt;=1,IF(N18="",Overview!$B$27,N18),IF(D18="","",IF(IF(K18=0,FALSE(),INDEX(F$2:F$29,K18)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K18=0,0,INDEX(F$2:F$29,K18)),IFERROR(LOOKUP(2,1/(M$2:M17=M18),P$2:P17),0)),1))))</f>
         <v/>
       </c>
       <c r="F18" s="16">
@@ -2284,7 +2333,7 @@
         </is>
       </c>
       <c r="O18" s="18">
-        <f>IF(OR(L18="",L18&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L18/Overview!$B$9,0))</f>
+        <f>IF(AND(Q18&lt;&gt;"",Q18&gt;0),ROUNDUP(Q18/Overview!$B$31,0),IF(OR(L18="",L18&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L18/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P18" s="16">
@@ -2311,7 +2360,7 @@
         <v/>
       </c>
       <c r="E19" s="16">
-        <f>IF(G19&gt;=1,IF(N19="",Overview!$B$27,N19),IF(D19="","",IF(IF(K19=0,FALSE(),INDEX(F$2:F$24,K19)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K19=0,0,INDEX(F$2:F$24,K19)),IFERROR(LOOKUP(2,1/(M$2:M18=M19),P$2:P18),0)),1))))</f>
+        <f>IF(G19&gt;=1,IF(N19="",Overview!$B$27,N19),IF(D19="","",IF(IF(K19=0,FALSE(),INDEX(F$2:F$29,K19)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K19=0,0,INDEX(F$2:F$29,K19)),IFERROR(LOOKUP(2,1/(M$2:M18=M19),P$2:P18),0)),1))))</f>
         <v/>
       </c>
       <c r="F19" s="16">
@@ -2350,7 +2399,7 @@
         </is>
       </c>
       <c r="O19" s="18">
-        <f>IF(OR(L19="",L19&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L19/Overview!$B$9,0))</f>
+        <f>IF(AND(Q19&lt;&gt;"",Q19&gt;0),ROUNDUP(Q19/Overview!$B$31,0),IF(OR(L19="",L19&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L19/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P19" s="16">
@@ -2369,7 +2418,7 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Settings: ~95%. Plan &amp; billing toast; Go Premium → /home#premium.</t>
+          <t>Account settings: Done. Billing entry peeled → leftover task 28 (1h); checkout → Payments 20.</t>
         </is>
       </c>
       <c r="D20" s="18">
@@ -2377,7 +2426,7 @@
         <v/>
       </c>
       <c r="E20" s="16">
-        <f>IF(G20&gt;=1,IF(N20="",Overview!$B$27,N20),IF(D20="","",IF(IF(K20=0,FALSE(),INDEX(F$2:F$24,K20)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K20=0,0,INDEX(F$2:F$24,K20)),IFERROR(LOOKUP(2,1/(M$2:M19=M20),P$2:P19),0)),1))))</f>
+        <f>IF(G20&gt;=1,IF(N20="",Overview!$B$27,N20),IF(D20="","",IF(IF(K20=0,FALSE(),INDEX(F$2:F$29,K20)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K20=0,0,INDEX(F$2:F$29,K20)),IFERROR(LOOKUP(2,1/(M$2:M19=M20),P$2:P19),0)),1))))</f>
         <v/>
       </c>
       <c r="F20" s="16">
@@ -2385,7 +2434,7 @@
         <v/>
       </c>
       <c r="G20" s="22" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H20" s="12">
         <f>IF(G20&gt;=1,"Done",IF(O20="","Scope pending",IF(E20="","Waiting on dependency",IF(G20&gt;0,"In progress","Planned"))))</f>
@@ -2410,9 +2459,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N20" s="16" t="n"/>
+      <c r="N20" s="16" t="n">
+        <v>46304</v>
+      </c>
       <c r="O20" s="18">
-        <f>IF(OR(L20="",L20&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L20/Overview!$B$9,0))</f>
+        <f>IF(AND(Q20&lt;&gt;"",Q20&gt;0),ROUNDUP(Q20/Overview!$B$31,0),IF(OR(L20="",L20&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L20/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P20" s="16">
@@ -2439,7 +2490,7 @@
         <v/>
       </c>
       <c r="E21" s="16">
-        <f>IF(G21&gt;=1,IF(N21="",Overview!$B$27,N21),IF(D21="","",IF(IF(K21=0,FALSE(),INDEX(F$2:F$24,K21)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K21=0,0,INDEX(F$2:F$24,K21)),IFERROR(LOOKUP(2,1/(M$2:M20=M21),P$2:P20),0)),1))))</f>
+        <f>IF(G21&gt;=1,IF(N21="",Overview!$B$27,N21),IF(D21="","",IF(IF(K21=0,FALSE(),INDEX(F$2:F$29,K21)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K21=0,0,INDEX(F$2:F$29,K21)),IFERROR(LOOKUP(2,1/(M$2:M20=M21),P$2:P20),0)),1))))</f>
         <v/>
       </c>
       <c r="F21" s="16">
@@ -2472,7 +2523,7 @@
       </c>
       <c r="N21" s="16" t="n"/>
       <c r="O21" s="18">
-        <f>IF(OR(L21="",L21&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L21/Overview!$B$9,0))</f>
+        <f>IF(AND(Q21&lt;&gt;"",Q21&gt;0),ROUNDUP(Q21/Overview!$B$31,0),IF(OR(L21="",L21&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L21/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P21" s="16">
@@ -2499,7 +2550,7 @@
         <v/>
       </c>
       <c r="E22" s="16">
-        <f>IF(G22&gt;=1,IF(N22="",Overview!$B$27,N22),IF(D22="","",IF(IF(K22=0,FALSE(),INDEX(F$2:F$24,K22)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K22=0,0,INDEX(F$2:F$24,K22)),IFERROR(LOOKUP(2,1/(M$2:M21=M22),P$2:P21),0)),1))))</f>
+        <f>IF(G22&gt;=1,IF(N22="",Overview!$B$27,N22),IF(D22="","",IF(IF(K22=0,FALSE(),INDEX(F$2:F$29,K22)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K22=0,0,INDEX(F$2:F$29,K22)),IFERROR(LOOKUP(2,1/(M$2:M21=M22),P$2:P21),0)),1))))</f>
         <v/>
       </c>
       <c r="F22" s="16">
@@ -2532,7 +2583,7 @@
       </c>
       <c r="N22" s="16" t="n"/>
       <c r="O22" s="18">
-        <f>IF(OR(L22="",L22&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L22/Overview!$B$9,0))</f>
+        <f>IF(AND(Q22&lt;&gt;"",Q22&gt;0),ROUNDUP(Q22/Overview!$B$31,0),IF(OR(L22="",L22&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L22/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P22" s="16">
@@ -2551,7 +2602,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>E2E QA: backlog from audit — #experts CTAs, Premium loops, rate-match, Socket.IO, JWT, empty british-coins chip.</t>
+          <t>E2E QA after leftover 28 + Premium 5 (25/26 done). Also: british-coins empty chip, other-apps Coming soon (intentional).</t>
         </is>
       </c>
       <c r="D23" s="18">
@@ -2559,7 +2610,7 @@
         <v/>
       </c>
       <c r="E23" s="16">
-        <f>IF(G23&gt;=1,IF(N23="",Overview!$B$27,N23),IF(D23="","",IF(COUNTIF(H2:H22,"Scope pending")+COUNTIF(H2:H22,"Waiting on dependency")+IF(G24&lt;1,IF(F24="",1,0),0)&gt;0,"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,MAX(F2:F22,F24)),1))))</f>
+        <f>IF(G23&gt;=1,IF(N23="",Overview!$B$27,N23),IF(D23="","",IF(COUNTIF(H2:H22,"Scope pending")+COUNTIF(H2:H22,"Waiting on dependency")+COUNTIF(H24:H29,"Scope pending")+COUNTIF(H24:H29,"Waiting on dependency")+COUNTIF(H24:H29,"In progress")+COUNTIF(H24:H29,"Planned")&gt;0,"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,MAX(F2:F22,F24:F29)),1))))</f>
         <v/>
       </c>
       <c r="F23" s="16">
@@ -2594,7 +2645,7 @@
       </c>
       <c r="N23" s="16" t="n"/>
       <c r="O23" s="18">
-        <f>IF(OR(L23="",L23&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L23/Overview!$B$9,0))</f>
+        <f>IF(AND(Q23&lt;&gt;"",Q23&gt;0),ROUNDUP(Q23/Overview!$B$31,0),IF(OR(L23="",L23&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L23/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P23" s="16">
@@ -2621,7 +2672,7 @@
         <v/>
       </c>
       <c r="E24" s="16">
-        <f>IF(G24&gt;=1,IF(N24="",Overview!$B$27,N24),IF(D24="","",IF(IF(K24=0,FALSE(),INDEX(F$2:F$24,K24)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K24=0,0,INDEX(F$2:F$24,K24)),IFERROR(LOOKUP(2,1/(M$2:M23=M24),P$2:P23),0)),1))))</f>
+        <f>IF(G24&gt;=1,IF(N24="",Overview!$B$27,N24),IF(D24="","",IF(IF(K24=0,FALSE(),INDEX(F$2:F$29,K24)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K24=0,0,INDEX(F$2:F$29,K24)),IFERROR(LOOKUP(2,1/(M$2:M23=M24),P$2:P23),0)),1))))</f>
         <v/>
       </c>
       <c r="F24" s="16">
@@ -2653,12 +2704,330 @@
         <v>46300</v>
       </c>
       <c r="O24" s="18">
-        <f>IF(OR(L24="",L24&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L24/Overview!$B$9,0))</f>
+        <f>IF(AND(Q24&lt;&gt;"",Q24&gt;0),ROUNDUP(Q24/Overview!$B$31,0),IF(OR(L24="",L24&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L24/Overview!$B$9,0)))</f>
         <v/>
       </c>
       <c r="P24" s="16">
         <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M23=M24),P$2:P23),0),IF(G24&gt;=1,0,IF(F24="",0,F24)))</f>
         <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Landing Expert CTAs: Done — Get Expert’s opinion? / View all → /auth?next=/experts</t>
+        </is>
+      </c>
+      <c r="D25" s="12">
+        <f>IF(G25&gt;=1,0,IF(O25="","",ROUNDUP(O25*(1-G25),0)))</f>
+        <v/>
+      </c>
+      <c r="E25" s="12">
+        <f>IF(G25&gt;=1,IF(N25="",Overview!$B$27,N25),IF(D25="","",IF(IF(K25=0,FALSE(),INDEX(F$2:F$29,K25)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K25=0,0,INDEX(F$2:F$29,K25)),IFERROR(LOOKUP(2,1/(M$2:M24=M25),P$2:P24),0)),1))))</f>
+        <v/>
+      </c>
+      <c r="F25" s="12">
+        <f>IF(G25&gt;=1,E25,IF(E25="","",WORKDAY(E25,D25-1)))</f>
+        <v/>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="12">
+        <f>IF(G25&gt;=1,"Done",IF(O25="","Scope pending",IF(E25="","Waiting on dependency",IF(G25&gt;0,"In progress","Planned"))))</f>
+        <v/>
+      </c>
+      <c r="I25" s="12">
+        <f>IF(E25="","",INT((E25-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="J25" s="12">
+        <f>IF(F25="","",INT((F25-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="K25" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N25" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O25" s="12">
+        <f>IF(AND(Q25&lt;&gt;"",Q25&gt;0),ROUNDUP(Q25/Overview!$B$31,0),IF(OR(L25="",L25&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L25/Overview!$B$9,0)))</f>
+        <v/>
+      </c>
+      <c r="P25" s="12">
+        <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M24=M25),P$2:P24),0),IF(G25&gt;=1,0,IF(F25="",0,F25)))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Identify rate-match: Done — Figma rate card (Stroke + Solid primary selected) + Message/Submit; dummy Feedback sent toast (no API).</t>
+        </is>
+      </c>
+      <c r="D26" s="12">
+        <f>IF(G26&gt;=1,0,IF(O26="","",ROUNDUP(O26*(1-G26),0)))</f>
+        <v/>
+      </c>
+      <c r="E26" s="12">
+        <f>IF(G26&gt;=1,IF(N26="",Overview!$B$27,N26),IF(D26="","",IF(IF(K26=0,FALSE(),INDEX(F$2:F$29,K26)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K26=0,0,INDEX(F$2:F$29,K26)),IFERROR(LOOKUP(2,1/(M$2:M25=M26),P$2:P25),0)),1))))</f>
+        <v/>
+      </c>
+      <c r="F26" s="12">
+        <f>IF(G26&gt;=1,E26,IF(E26="","",WORKDAY(E26,D26-1)))</f>
+        <v/>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="12">
+        <f>IF(G26&gt;=1,"Done",IF(O26="","Scope pending",IF(E26="","Waiting on dependency",IF(G26&gt;0,"In progress","Planned"))))</f>
+        <v/>
+      </c>
+      <c r="I26" s="12">
+        <f>IF(E26="","",INT((E26-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="J26" s="12">
+        <f>IF(F26="","",INT((F26-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="K26" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N26" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O26" s="12">
+        <f>IF(AND(Q26&lt;&gt;"",Q26&gt;0),ROUNDUP(Q26/Overview!$B$31,0),IF(OR(L26="",L26&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L26/Overview!$B$9,0)))</f>
+        <v/>
+      </c>
+      <c r="P26" s="12">
+        <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M25=M26),P$2:P25),0),IF(G26&gt;=1,0,IF(F26="",0,F26)))</f>
+        <v/>
+      </c>
+      <c r="Q26" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Experts Socket.IO: Done — socket.io-client → Experts host auth.userId; events trigger REST refresh / router.refresh. Poll kept as fallback.</t>
+        </is>
+      </c>
+      <c r="D27" s="12">
+        <f>IF(G27&gt;=1,0,IF(O27="","",ROUNDUP(O27*(1-G27),0)))</f>
+        <v/>
+      </c>
+      <c r="E27" s="12">
+        <f>IF(G27&gt;=1,IF(N27="",Overview!$B$27,N27),IF(D27="","",IF(IF(K27=0,FALSE(),INDEX(F$2:F$29,K27)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K27=0,0,INDEX(F$2:F$29,K27)),IFERROR(LOOKUP(2,1/(M$2:M26=M27),P$2:P26),0)),1))))</f>
+        <v/>
+      </c>
+      <c r="F27" s="12">
+        <f>IF(G27&gt;=1,E27,IF(E27="","",WORKDAY(E27,D27-1)))</f>
+        <v/>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="12">
+        <f>IF(G27&gt;=1,"Done",IF(O27="","Scope pending",IF(E27="","Waiting on dependency",IF(G27&gt;0,"In progress","Planned"))))</f>
+        <v/>
+      </c>
+      <c r="I27" s="12">
+        <f>IF(E27="","",INT((E27-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="J27" s="12">
+        <f>IF(F27="","",INT((F27-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N27" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O27" s="12">
+        <f>IF(AND(Q27&lt;&gt;"",Q27&gt;0),ROUNDUP(Q27/Overview!$B$31,0),IF(OR(L27="",L27&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L27/Overview!$B$9,0)))</f>
+        <v/>
+      </c>
+      <c r="P27" s="12">
+        <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M26=M27),P$2:P26),0),IF(G27&gt;=1,0,IF(F27="",0,F27)))</f>
+        <v/>
+      </c>
+      <c r="Q27" s="12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>(cancelled — was manage polish): Out of scope. Edit/rename private not on web. ID kept.</t>
+        </is>
+      </c>
+      <c r="D28" s="12">
+        <f>IF(G28&gt;=1,0,IF(O28="","",ROUNDUP(O28*(1-G28),0)))</f>
+        <v/>
+      </c>
+      <c r="E28" s="12">
+        <f>IF(G28&gt;=1,IF(N28="",Overview!$B$27,N28),IF(D28="","",IF(IF(K28=0,FALSE(),INDEX(F$2:F$29,K28)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K28=0,0,INDEX(F$2:F$29,K28)),IFERROR(LOOKUP(2,1/(M$2:M27=M28),P$2:P27),0)),1))))</f>
+        <v/>
+      </c>
+      <c r="F28" s="12">
+        <f>IF(G28&gt;=1,E28,IF(E28="","",WORKDAY(E28,D28-1)))</f>
+        <v/>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="12">
+        <f>IF(G28&gt;=1,"Done",IF(O28="","Scope pending",IF(E28="","Waiting on dependency",IF(G28&gt;0,"In progress","Planned"))))</f>
+        <v/>
+      </c>
+      <c r="I28" s="12">
+        <f>IF(E28="","",INT((E28-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="J28" s="12">
+        <f>IF(F28="","",INT((F28-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N28" s="24" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O28" s="12">
+        <f>IF(AND(Q28&lt;&gt;"",Q28&gt;0),ROUNDUP(Q28/Overview!$B$31,0),IF(OR(L28="",L28&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L28/Overview!$B$9,0)))</f>
+        <v/>
+      </c>
+      <c r="P28" s="12">
+        <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M27=M28),P$2:P27),0),IF(G28&gt;=1,0,IF(F28="",0,F28)))</f>
+        <v/>
+      </c>
+      <c r="Q28" s="12" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Leftovers (hours)</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Settings billing entry: Done — opens test Premium plans. Real gateway → Payments 20.</t>
+        </is>
+      </c>
+      <c r="D29" s="12">
+        <f>IF(G29&gt;=1,0,IF(O29="","",ROUNDUP(O29*(1-G29),0)))</f>
+        <v/>
+      </c>
+      <c r="E29" s="12">
+        <f>IF(G29&gt;=1,IF(N29="",Overview!$B$27,N29),IF(D29="","",IF(IF(K29=0,FALSE(),INDEX(F$2:F$29,K29)=""),"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,IF(K29=0,0,INDEX(F$2:F$29,K29)),IFERROR(LOOKUP(2,1/(M$2:M28=M29),P$2:P28),0)),1))))</f>
+        <v/>
+      </c>
+      <c r="F29" s="12">
+        <f>IF(G29&gt;=1,E29,IF(E29="","",WORKDAY(E29,D29-1)))</f>
+        <v/>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="12">
+        <f>IF(G29&gt;=1,"Done",IF(O29="","Scope pending",IF(E29="","Waiting on dependency",IF(G29&gt;0,"In progress","Planned"))))</f>
+        <v/>
+      </c>
+      <c r="I29" s="12">
+        <f>IF(E29="","",INT((E29-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="J29" s="12">
+        <f>IF(F29="","",INT((F29-Overview!$B$2)/7)+1)</f>
+        <v/>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="M29" s="12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N29" s="24" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O29" s="12">
+        <f>IF(AND(Q29&lt;&gt;"",Q29&gt;0),ROUNDUP(Q29/Overview!$B$31,0),IF(OR(L29="",L29&lt;=0,Overview!$B$9&lt;=0),"",ROUNDUP(L29/Overview!$B$9,0)))</f>
+        <v/>
+      </c>
+      <c r="P29" s="12">
+        <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M28=M29),P$2:P28),0),IF(G29&gt;=1,0,IF(F29="",0,F29)))</f>
+        <v/>
+      </c>
+      <c r="Q29" s="12" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2689,7 +3058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="12" min="1" max="1"/>
@@ -5556,6 +5925,316 @@
       </c>
       <c r="AC24" s="23">
         <f>IF(OR('Detailed Timeline'!$I23="",'Detailed Timeline'!$J23=""),"",IF(AND(26&gt;='Detailed Timeline'!$I23,26&lt;='Detailed Timeline'!$J23),"■",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12">
+        <f>'Detailed Timeline'!A25</f>
+        <v/>
+      </c>
+      <c r="B25" s="12">
+        <f>'Detailed Timeline'!B25</f>
+        <v/>
+      </c>
+      <c r="C25" s="12">
+        <f>'Detailed Timeline'!C25</f>
+        <v/>
+      </c>
+      <c r="D25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(1&gt;='Detailed Timeline'!$I25,1&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="E25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(2&gt;='Detailed Timeline'!$I25,2&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="F25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(3&gt;='Detailed Timeline'!$I25,3&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="G25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(4&gt;='Detailed Timeline'!$I25,4&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="H25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(5&gt;='Detailed Timeline'!$I25,5&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="I25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(6&gt;='Detailed Timeline'!$I25,6&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="J25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(7&gt;='Detailed Timeline'!$I25,7&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="K25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(8&gt;='Detailed Timeline'!$I25,8&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="L25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(9&gt;='Detailed Timeline'!$I25,9&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="M25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(10&gt;='Detailed Timeline'!$I25,10&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="N25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(11&gt;='Detailed Timeline'!$I25,11&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+      <c r="O25" s="12">
+        <f>IF(OR('Detailed Timeline'!$I25="",'Detailed Timeline'!$J25=""),"",IF(AND(12&gt;='Detailed Timeline'!$I25,12&lt;='Detailed Timeline'!$J25),"■",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12">
+        <f>'Detailed Timeline'!A26</f>
+        <v/>
+      </c>
+      <c r="B26" s="12">
+        <f>'Detailed Timeline'!B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="12">
+        <f>'Detailed Timeline'!C26</f>
+        <v/>
+      </c>
+      <c r="D26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(1&gt;='Detailed Timeline'!$I26,1&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="E26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(2&gt;='Detailed Timeline'!$I26,2&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="F26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(3&gt;='Detailed Timeline'!$I26,3&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="G26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(4&gt;='Detailed Timeline'!$I26,4&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="H26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(5&gt;='Detailed Timeline'!$I26,5&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="I26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(6&gt;='Detailed Timeline'!$I26,6&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="J26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(7&gt;='Detailed Timeline'!$I26,7&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="K26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(8&gt;='Detailed Timeline'!$I26,8&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="L26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(9&gt;='Detailed Timeline'!$I26,9&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="M26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(10&gt;='Detailed Timeline'!$I26,10&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="N26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(11&gt;='Detailed Timeline'!$I26,11&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+      <c r="O26" s="12">
+        <f>IF(OR('Detailed Timeline'!$I26="",'Detailed Timeline'!$J26=""),"",IF(AND(12&gt;='Detailed Timeline'!$I26,12&lt;='Detailed Timeline'!$J26),"■",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12">
+        <f>'Detailed Timeline'!A27</f>
+        <v/>
+      </c>
+      <c r="B27" s="12">
+        <f>'Detailed Timeline'!B27</f>
+        <v/>
+      </c>
+      <c r="C27" s="12">
+        <f>'Detailed Timeline'!C27</f>
+        <v/>
+      </c>
+      <c r="D27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(1&gt;='Detailed Timeline'!$I27,1&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="E27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(2&gt;='Detailed Timeline'!$I27,2&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="F27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(3&gt;='Detailed Timeline'!$I27,3&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="G27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(4&gt;='Detailed Timeline'!$I27,4&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="H27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(5&gt;='Detailed Timeline'!$I27,5&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="I27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(6&gt;='Detailed Timeline'!$I27,6&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="J27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(7&gt;='Detailed Timeline'!$I27,7&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="K27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(8&gt;='Detailed Timeline'!$I27,8&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="L27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(9&gt;='Detailed Timeline'!$I27,9&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="M27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(10&gt;='Detailed Timeline'!$I27,10&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="N27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(11&gt;='Detailed Timeline'!$I27,11&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+      <c r="O27" s="12">
+        <f>IF(OR('Detailed Timeline'!$I27="",'Detailed Timeline'!$J27=""),"",IF(AND(12&gt;='Detailed Timeline'!$I27,12&lt;='Detailed Timeline'!$J27),"■",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12">
+        <f>'Detailed Timeline'!A28</f>
+        <v/>
+      </c>
+      <c r="B28" s="12">
+        <f>'Detailed Timeline'!B28</f>
+        <v/>
+      </c>
+      <c r="C28" s="12">
+        <f>'Detailed Timeline'!C28</f>
+        <v/>
+      </c>
+      <c r="D28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(1&gt;='Detailed Timeline'!$I28,1&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="E28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(2&gt;='Detailed Timeline'!$I28,2&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="F28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(3&gt;='Detailed Timeline'!$I28,3&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="G28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(4&gt;='Detailed Timeline'!$I28,4&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="H28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(5&gt;='Detailed Timeline'!$I28,5&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="I28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(6&gt;='Detailed Timeline'!$I28,6&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="J28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(7&gt;='Detailed Timeline'!$I28,7&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="K28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(8&gt;='Detailed Timeline'!$I28,8&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="L28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(9&gt;='Detailed Timeline'!$I28,9&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="M28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(10&gt;='Detailed Timeline'!$I28,10&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="N28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(11&gt;='Detailed Timeline'!$I28,11&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+      <c r="O28" s="12">
+        <f>IF(OR('Detailed Timeline'!$I28="",'Detailed Timeline'!$J28=""),"",IF(AND(12&gt;='Detailed Timeline'!$I28,12&lt;='Detailed Timeline'!$J28),"■",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12">
+        <f>'Detailed Timeline'!A29</f>
+        <v/>
+      </c>
+      <c r="B29" s="12">
+        <f>'Detailed Timeline'!B29</f>
+        <v/>
+      </c>
+      <c r="C29" s="12">
+        <f>'Detailed Timeline'!C29</f>
+        <v/>
+      </c>
+      <c r="D29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(1&gt;='Detailed Timeline'!$I29,1&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="E29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(2&gt;='Detailed Timeline'!$I29,2&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="F29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(3&gt;='Detailed Timeline'!$I29,3&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="G29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(4&gt;='Detailed Timeline'!$I29,4&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="H29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(5&gt;='Detailed Timeline'!$I29,5&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="I29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(6&gt;='Detailed Timeline'!$I29,6&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="J29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(7&gt;='Detailed Timeline'!$I29,7&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="K29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(8&gt;='Detailed Timeline'!$I29,8&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="L29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(9&gt;='Detailed Timeline'!$I29,9&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="M29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(10&gt;='Detailed Timeline'!$I29,10&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="N29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(11&gt;='Detailed Timeline'!$I29,11&lt;='Detailed Timeline'!$J29),"■",""))</f>
+        <v/>
+      </c>
+      <c r="O29" s="12">
+        <f>IF(OR('Detailed Timeline'!$I29="",'Detailed Timeline'!$J29=""),"",IF(AND(12&gt;='Detailed Timeline'!$I29,12&lt;='Detailed Timeline'!$J29),"■",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: sync INDEX, AGENTS, checklist, bug tracker and timeline with shipped fixes
- INDEX.md: notes for identify scan counting, previews, match list, drawer, multi-select
  collections, rate card, home loading and SEO files.
- docs/bug-tracker.html: ClickUp tickets marked fixed locally (14yn59xnnj3, xntxu,
  xnu85, xnu8r, xnujt, xnuqx, xnv6h, xnvhy, xnvjx, xnvme) and xnvpf closed as a
  backend issue.
- AGENTS.md, PAGES-CHECKLIST.md and the timeline html/xlsx/test refreshed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/coinzy-web-timeline.xlsx
+++ b/coinzy-web-timeline.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Parallel AI agents; screen tasks use screens/day; leftovers use hours (see Hours col + hours/day).</t>
+          <t>Parallel AI agents; screen tasks use screens/day; leftovers + QA bug backlog use hours. Bug ETA from docs/bug-tracker.html velocity.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Sync 22 (14 Oct 2026): Hour leftovers closed (24–26/28 done, 27 cancelled). Next: E2E QA task 22. Deferred (not QA blockers): Payments 20 real gateway; Premium task 5 JWT entitlement (test cookie OK for QA).</t>
+          <t>Sync 23 (28 Oct 2026): Critical path = ClickUp web bugs. Velocity 34 pts/day (13 fixed today). 63 open (147 pts) → calendar ETA 2026-11-02 (~5d); workday finish ~2026-11-04. Task 22 = E2E+bug backlog 40h. Deferred (not QA blockers): Payments 20; Premium JWT on task 5.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Hour leftovers: none open. Ready for E2E QA (task 22).</t>
+          <t>Bug ETA assumes today’s burst holds. Half-pace (~17 pts/day) → ~2026-11-06. See docs/bug-tracker.html.</t>
         </is>
       </c>
     </row>
@@ -1070,8 +1070,8 @@
           <t>Forecast from (edit)</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n">
-        <v>46309</v>
+      <c r="B27" s="15">
+        <v>46323</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="13">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Premium experience: ~95% test multi-plan purchase (coinzy_premium cookie). Real gateway → Payments 20.</t>
+          <t>Premium experience: ~95% test multi-plan purchase (coinzy_premium cookie). JWT + Payments 20 deferred/unscheduled (not QA blocker).</t>
         </is>
       </c>
       <c r="D6" s="18">
@@ -1553,9 +1553,7 @@
       <c r="K6" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="L6" s="18" t="n">
-        <v>4</v>
-      </c>
+      <c r="L6" s="18"/>
       <c r="M6" s="12" t="inlineStr">
         <is>
           <t>B</t>
@@ -2602,7 +2600,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>E2E QA after leftover 28 + Premium 5 (25/26 done). Also: british-coins empty chip, other-apps Coming soon (intentional).</t>
+          <t>E2E QA + ClickUp bug backlog: 13 fixed / 34 pts on 2026-10-28; 63 open / 147 pts → ~5 agent days (40h) at 34 pts/day. british-coins empty chip + other-apps Coming soon intentional.</t>
         </is>
       </c>
       <c r="D23" s="18">
@@ -2610,8 +2608,7 @@
         <v/>
       </c>
       <c r="E23" s="16">
-        <f>IF(G23&gt;=1,IF(N23="",Overview!$B$27,N23),IF(D23="","",IF(COUNTIF(H2:H22,"Scope pending")+COUNTIF(H2:H22,"Waiting on dependency")+COUNTIF(H24:H29,"Scope pending")+COUNTIF(H24:H29,"Waiting on dependency")+COUNTIF(H24:H29,"In progress")+COUNTIF(H24:H29,"Planned")&gt;0,"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,MAX(F2:F22,F24:F29)),1))))</f>
-        <v/>
+        <f>IF(G23&gt;=1,IF(N23="",Overview!$B$27,N23),IF(D23="","",IF(COUNTIF(H2:H22,"Waiting on dependency")+COUNTIF(H24:H29,"Waiting on dependency")&gt;0,"",WORKDAY(MAX(Overview!$B$2-1,Overview!$B$27-1,MAX(F2:F22,F24:F29)),1))))</f>
       </c>
       <c r="F23" s="16">
         <f>IF(G23&gt;=1,E23,IF(E23="","",WORKDAY(E23,D23-1)))</f>
@@ -2635,9 +2632,7 @@
       <c r="K23" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="18" t="n">
-        <v>6</v>
-      </c>
+      <c r="L23" s="18"/>
       <c r="M23" s="12" t="inlineStr">
         <is>
           <t>QA</t>
@@ -2651,6 +2646,9 @@
       <c r="P23" s="16">
         <f>MAX(IFERROR(LOOKUP(2,1/(M$2:M22=M23),P$2:P22),0),IF(G23&gt;=1,0,IF(F23="",0,F23)))</f>
         <v/>
+      </c>
+      <c r="Q23" s="12">
+        <v>40</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="13">

</xml_diff>